<commit_message>
Charges perso : mode de paiement, compte débité et jour du mois
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KqkJNWVZSWN9upSPoUaH5h
</commit_message>
<xml_diff>
--- a/suivi_comptes_example.xlsx
+++ b/suivi_comptes_example.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="166">
   <si>
     <t xml:space="preserve">Synthèse mensuelle</t>
   </si>
@@ -4454,13 +4454,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="9"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4492,6 +4495,15 @@
       <c r="F4" s="4" t="s">
         <v>89</v>
       </c>
+      <c r="G4" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
@@ -4513,6 +4525,15 @@
         <f aca="false">IF(A5="","",IFERROR(E5/INDEX(Paramètres!$E$4:$E$7,MATCH(D5,Paramètres!$D$4:$D$7,0)),0))</f>
         <v>35</v>
       </c>
+      <c r="G5" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="H5" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="I5" s="13" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
@@ -4534,6 +4555,13 @@
         <f aca="false">IF(A6="","",IFERROR(E6/INDEX(Paramètres!$E$4:$E$7,MATCH(D6,Paramètres!$D$4:$D$7,0)),0))</f>
         <v>40</v>
       </c>
+      <c r="G6" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="I6" s="13"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
@@ -4554,6 +4582,15 @@
       <c r="F7" s="6" t="n">
         <f aca="false">IF(A7="","",IFERROR(E7/INDEX(Paramètres!$E$4:$E$7,MATCH(D7,Paramètres!$D$4:$D$7,0)),0))</f>
         <v>11</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="H7" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="I7" s="13" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4566,6 +4603,9 @@
         <f aca="false">IF(A8="","",IFERROR(E8/INDEX(Paramètres!$E$4:$E$7,MATCH(D8,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
+      <c r="I8" s="13"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13"/>
@@ -4577,6 +4617,9 @@
         <f aca="false">IF(A9="","",IFERROR(E9/INDEX(Paramètres!$E$4:$E$7,MATCH(D9,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G9" s="13"/>
+      <c r="H9" s="13"/>
+      <c r="I9" s="13"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13"/>
@@ -4588,6 +4631,9 @@
         <f aca="false">IF(A10="","",IFERROR(E10/INDEX(Paramètres!$E$4:$E$7,MATCH(D10,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="13"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13"/>
@@ -4599,6 +4645,9 @@
         <f aca="false">IF(A11="","",IFERROR(E11/INDEX(Paramètres!$E$4:$E$7,MATCH(D11,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="13"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13"/>
@@ -4610,6 +4659,9 @@
         <f aca="false">IF(A12="","",IFERROR(E12/INDEX(Paramètres!$E$4:$E$7,MATCH(D12,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="13"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13"/>
@@ -4621,6 +4673,9 @@
         <f aca="false">IF(A13="","",IFERROR(E13/INDEX(Paramètres!$E$4:$E$7,MATCH(D13,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="13"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13"/>
@@ -4632,6 +4687,9 @@
         <f aca="false">IF(A14="","",IFERROR(E14/INDEX(Paramètres!$E$4:$E$7,MATCH(D14,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G14" s="13"/>
+      <c r="H14" s="13"/>
+      <c r="I14" s="13"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13"/>
@@ -4643,6 +4701,9 @@
         <f aca="false">IF(A15="","",IFERROR(E15/INDEX(Paramètres!$E$4:$E$7,MATCH(D15,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="13"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13"/>
@@ -4654,6 +4715,9 @@
         <f aca="false">IF(A16="","",IFERROR(E16/INDEX(Paramètres!$E$4:$E$7,MATCH(D16,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
+      <c r="I16" s="13"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13"/>
@@ -4665,6 +4729,9 @@
         <f aca="false">IF(A17="","",IFERROR(E17/INDEX(Paramètres!$E$4:$E$7,MATCH(D17,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G17" s="13"/>
+      <c r="H17" s="13"/>
+      <c r="I17" s="13"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13"/>
@@ -4676,6 +4743,9 @@
         <f aca="false">IF(A18="","",IFERROR(E18/INDEX(Paramètres!$E$4:$E$7,MATCH(D18,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13"/>
+      <c r="I18" s="13"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13"/>
@@ -4687,6 +4757,9 @@
         <f aca="false">IF(A19="","",IFERROR(E19/INDEX(Paramètres!$E$4:$E$7,MATCH(D19,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="13"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13"/>
@@ -4698,6 +4771,9 @@
         <f aca="false">IF(A20="","",IFERROR(E20/INDEX(Paramètres!$E$4:$E$7,MATCH(D20,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G20" s="13"/>
+      <c r="H20" s="13"/>
+      <c r="I20" s="13"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13"/>
@@ -4709,6 +4785,9 @@
         <f aca="false">IF(A21="","",IFERROR(E21/INDEX(Paramètres!$E$4:$E$7,MATCH(D21,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G21" s="13"/>
+      <c r="H21" s="13"/>
+      <c r="I21" s="13"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13"/>
@@ -4720,6 +4799,9 @@
         <f aca="false">IF(A22="","",IFERROR(E22/INDEX(Paramètres!$E$4:$E$7,MATCH(D22,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G22" s="13"/>
+      <c r="H22" s="13"/>
+      <c r="I22" s="13"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13"/>
@@ -4731,6 +4813,9 @@
         <f aca="false">IF(A23="","",IFERROR(E23/INDEX(Paramètres!$E$4:$E$7,MATCH(D23,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G23" s="13"/>
+      <c r="H23" s="13"/>
+      <c r="I23" s="13"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13"/>
@@ -4742,6 +4827,9 @@
         <f aca="false">IF(A24="","",IFERROR(E24/INDEX(Paramètres!$E$4:$E$7,MATCH(D24,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G24" s="13"/>
+      <c r="H24" s="13"/>
+      <c r="I24" s="13"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13"/>
@@ -4753,6 +4841,9 @@
         <f aca="false">IF(A25="","",IFERROR(E25/INDEX(Paramètres!$E$4:$E$7,MATCH(D25,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G25" s="13"/>
+      <c r="H25" s="13"/>
+      <c r="I25" s="13"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13"/>
@@ -4764,6 +4855,9 @@
         <f aca="false">IF(A26="","",IFERROR(E26/INDEX(Paramètres!$E$4:$E$7,MATCH(D26,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G26" s="13"/>
+      <c r="H26" s="13"/>
+      <c r="I26" s="13"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13"/>
@@ -4775,6 +4869,9 @@
         <f aca="false">IF(A27="","",IFERROR(E27/INDEX(Paramètres!$E$4:$E$7,MATCH(D27,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G27" s="13"/>
+      <c r="H27" s="13"/>
+      <c r="I27" s="13"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13"/>
@@ -4786,6 +4883,9 @@
         <f aca="false">IF(A28="","",IFERROR(E28/INDEX(Paramètres!$E$4:$E$7,MATCH(D28,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G28" s="13"/>
+      <c r="H28" s="13"/>
+      <c r="I28" s="13"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="13"/>
@@ -4797,6 +4897,9 @@
         <f aca="false">IF(A29="","",IFERROR(E29/INDEX(Paramètres!$E$4:$E$7,MATCH(D29,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G29" s="13"/>
+      <c r="H29" s="13"/>
+      <c r="I29" s="13"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13"/>
@@ -4808,6 +4911,9 @@
         <f aca="false">IF(A30="","",IFERROR(E30/INDEX(Paramètres!$E$4:$E$7,MATCH(D30,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G30" s="13"/>
+      <c r="H30" s="13"/>
+      <c r="I30" s="13"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13"/>
@@ -4819,6 +4925,9 @@
         <f aca="false">IF(A31="","",IFERROR(E31/INDEX(Paramètres!$E$4:$E$7,MATCH(D31,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G31" s="13"/>
+      <c r="H31" s="13"/>
+      <c r="I31" s="13"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13"/>
@@ -4830,6 +4939,9 @@
         <f aca="false">IF(A32="","",IFERROR(E32/INDEX(Paramètres!$E$4:$E$7,MATCH(D32,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G32" s="13"/>
+      <c r="H32" s="13"/>
+      <c r="I32" s="13"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13"/>
@@ -4841,6 +4953,9 @@
         <f aca="false">IF(A33="","",IFERROR(E33/INDEX(Paramètres!$E$4:$E$7,MATCH(D33,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G33" s="13"/>
+      <c r="H33" s="13"/>
+      <c r="I33" s="13"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13"/>
@@ -4852,6 +4967,9 @@
         <f aca="false">IF(A34="","",IFERROR(E34/INDEX(Paramètres!$E$4:$E$7,MATCH(D34,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G34" s="13"/>
+      <c r="H34" s="13"/>
+      <c r="I34" s="13"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13"/>
@@ -4863,6 +4981,9 @@
         <f aca="false">IF(A35="","",IFERROR(E35/INDEX(Paramètres!$E$4:$E$7,MATCH(D35,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G35" s="13"/>
+      <c r="H35" s="13"/>
+      <c r="I35" s="13"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13"/>
@@ -4874,6 +4995,9 @@
         <f aca="false">IF(A36="","",IFERROR(E36/INDEX(Paramètres!$E$4:$E$7,MATCH(D36,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G36" s="13"/>
+      <c r="H36" s="13"/>
+      <c r="I36" s="13"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13"/>
@@ -4885,6 +5009,9 @@
         <f aca="false">IF(A37="","",IFERROR(E37/INDEX(Paramètres!$E$4:$E$7,MATCH(D37,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G37" s="13"/>
+      <c r="H37" s="13"/>
+      <c r="I37" s="13"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13"/>
@@ -4896,6 +5023,9 @@
         <f aca="false">IF(A38="","",IFERROR(E38/INDEX(Paramètres!$E$4:$E$7,MATCH(D38,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G38" s="13"/>
+      <c r="H38" s="13"/>
+      <c r="I38" s="13"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="13"/>
@@ -4907,6 +5037,9 @@
         <f aca="false">IF(A39="","",IFERROR(E39/INDEX(Paramètres!$E$4:$E$7,MATCH(D39,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G39" s="13"/>
+      <c r="H39" s="13"/>
+      <c r="I39" s="13"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="13"/>
@@ -4918,6 +5051,9 @@
         <f aca="false">IF(A40="","",IFERROR(E40/INDEX(Paramètres!$E$4:$E$7,MATCH(D40,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G40" s="13"/>
+      <c r="H40" s="13"/>
+      <c r="I40" s="13"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="13"/>
@@ -4929,6 +5065,9 @@
         <f aca="false">IF(A41="","",IFERROR(E41/INDEX(Paramètres!$E$4:$E$7,MATCH(D41,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G41" s="13"/>
+      <c r="H41" s="13"/>
+      <c r="I41" s="13"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="13"/>
@@ -4940,6 +5079,9 @@
         <f aca="false">IF(A42="","",IFERROR(E42/INDEX(Paramètres!$E$4:$E$7,MATCH(D42,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G42" s="13"/>
+      <c r="H42" s="13"/>
+      <c r="I42" s="13"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="13"/>
@@ -4951,6 +5093,9 @@
         <f aca="false">IF(A43="","",IFERROR(E43/INDEX(Paramètres!$E$4:$E$7,MATCH(D43,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G43" s="13"/>
+      <c r="H43" s="13"/>
+      <c r="I43" s="13"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="13"/>
@@ -4962,6 +5107,9 @@
         <f aca="false">IF(A44="","",IFERROR(E44/INDEX(Paramètres!$E$4:$E$7,MATCH(D44,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
       </c>
+      <c r="G44" s="13"/>
+      <c r="H44" s="13"/>
+      <c r="I44" s="13"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="22" t="s">
@@ -4973,7 +5121,15 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="4">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G44" type="list">
+      <formula1>"Prélèvement,Carte,Chèque,Espèces,Virement"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H44" type="list">
+      <formula1>Comptes!$A$5:$A$14</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B44" type="list">
       <formula1>Paramètres!$B$4:$B$5</formula1>
       <formula2>0</formula2>

</xml_diff>

<commit_message>
Exemple d'électricité sur deux comptes joints
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KqkJNWVZSWN9upSPoUaH5h
</commit_message>
<xml_diff>
--- a/suivi_comptes_example.xlsx
+++ b/suivi_comptes_example.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="167">
   <si>
     <t xml:space="preserve">Synthèse mensuelle</t>
   </si>
@@ -337,13 +337,16 @@
     <t xml:space="preserve">Taxe foncière</t>
   </si>
   <si>
-    <t xml:space="preserve">Électricité / gaz</t>
+    <t xml:space="preserve">Électricité maison</t>
   </si>
   <si>
     <t xml:space="preserve">Énergie</t>
   </si>
   <si>
     <t xml:space="preserve">Variable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Électricité garage / local</t>
   </si>
   <si>
     <t xml:space="preserve">Internet / box</t>
@@ -1142,7 +1145,7 @@
       </c>
       <c r="C5" s="6" t="n">
         <f aca="false">SUM(E$13:E$22)</f>
-        <v>1404.28586025397</v>
+        <v>1424.28586025397</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">IF(Paramètres!$B$6="",0,IFERROR(INDEX($C$13:$C$22,MATCH(Paramètres!$B$6,$A$13:$A$22,0)),0))</f>
@@ -1150,15 +1153,15 @@
       </c>
       <c r="E5" s="6" t="n">
         <f aca="false">C5+D5</f>
-        <v>1404.28586025397</v>
+        <v>1424.28586025397</v>
       </c>
       <c r="F5" s="7" t="n">
         <f aca="false">IF(B5=0,0,E5/B5)</f>
-        <v>0.585119108439156</v>
+        <v>0.593452441772489</v>
       </c>
       <c r="G5" s="6" t="n">
         <f aca="false">IF(Paramètres!$B$6="",0,IFERROR(INDEX($J$13:$J$22,MATCH(Paramètres!$B$6,$A$13:$A$22,0)),0))</f>
-        <v>995.714139746026</v>
+        <v>975.714139746026</v>
       </c>
       <c r="H5" s="6" t="n">
         <f aca="false">IF(Paramètres!B$15="Forfait",Paramètres!B$16,SUMIFS('Charges perso'!$F$5:$F$44,'Charges perso'!$B$5:$B$44,A5))</f>
@@ -1166,15 +1169,15 @@
       </c>
       <c r="I5" s="6" t="n">
         <f aca="false">G5-H5</f>
-        <v>909.714139746026</v>
+        <v>889.714139746026</v>
       </c>
       <c r="J5" s="6" t="n">
         <f aca="false">MAX(0,IF(Paramètres!B$17="Pourcentage",Paramètres!B$18*MAX(0,I5),Paramètres!B$19))</f>
-        <v>272.914241923808</v>
+        <v>266.914241923808</v>
       </c>
       <c r="K5" s="6" t="n">
         <f aca="false">I5-J5</f>
-        <v>636.799897822218</v>
+        <v>622.799897822218</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1188,7 +1191,7 @@
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">SUM(F$13:F$22)</f>
-        <v>1199.71413974603</v>
+        <v>1219.71413974603</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">IF(Paramètres!$B$7="",0,IFERROR(INDEX($C$13:$C$22,MATCH(Paramètres!$B$7,$A$13:$A$22,0)),0))</f>
@@ -1196,15 +1199,15 @@
       </c>
       <c r="E6" s="6" t="n">
         <f aca="false">C6+D6</f>
-        <v>1227.71413974603</v>
+        <v>1247.71413974603</v>
       </c>
       <c r="F6" s="7" t="n">
         <f aca="false">IF(B6=0,0,E6/B6)</f>
-        <v>0.646165336708435</v>
+        <v>0.656691652497908</v>
       </c>
       <c r="G6" s="6" t="n">
         <f aca="false">IF(Paramètres!$B$7="",0,IFERROR(INDEX($J$13:$J$22,MATCH(Paramètres!$B$7,$A$13:$A$22,0)),0))</f>
-        <v>672.285860253974</v>
+        <v>652.285860253974</v>
       </c>
       <c r="H6" s="6" t="n">
         <f aca="false">IF(Paramètres!C$15="Forfait",Paramètres!C$16,SUMIFS('Charges perso'!$F$5:$F$44,'Charges perso'!$B$5:$B$44,A6))</f>
@@ -1212,7 +1215,7 @@
       </c>
       <c r="I6" s="6" t="n">
         <f aca="false">G6-H6</f>
-        <v>322.285860253974</v>
+        <v>302.285860253974</v>
       </c>
       <c r="J6" s="6" t="n">
         <f aca="false">MAX(0,IF(Paramètres!C$17="Pourcentage",Paramètres!C$18*MAX(0,I6),Paramètres!C$19))</f>
@@ -1220,7 +1223,7 @@
       </c>
       <c r="K6" s="6" t="n">
         <f aca="false">I6-J6</f>
-        <v>122.285860253974</v>
+        <v>102.285860253974</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1233,7 +1236,7 @@
       </c>
       <c r="C7" s="9" t="n">
         <f aca="false">SUM(C5:C6)</f>
-        <v>2604</v>
+        <v>2644</v>
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">SUM(D5:D6)</f>
@@ -1241,15 +1244,15 @@
       </c>
       <c r="E7" s="9" t="n">
         <f aca="false">SUM(E5:E6)</f>
-        <v>2632</v>
+        <v>2672</v>
       </c>
       <c r="F7" s="10" t="n">
         <f aca="false">IF(B7=0,0,E7/B7)</f>
-        <v>0.612093023255814</v>
+        <v>0.621395348837209</v>
       </c>
       <c r="G7" s="9" t="n">
         <f aca="false">SUM(G5:G6)</f>
-        <v>1668</v>
+        <v>1628</v>
       </c>
       <c r="H7" s="9" t="n">
         <f aca="false">SUM(H5:H6)</f>
@@ -1257,15 +1260,15 @@
       </c>
       <c r="I7" s="9" t="n">
         <f aca="false">SUM(I5:I6)</f>
-        <v>1232</v>
+        <v>1192</v>
       </c>
       <c r="J7" s="9" t="n">
         <f aca="false">SUM(J5:J6)</f>
-        <v>472.914241923808</v>
+        <v>466.914241923808</v>
       </c>
       <c r="K7" s="9" t="n">
         <f aca="false">SUM(K5:K6)</f>
-        <v>759.085758076192</v>
+        <v>725.085758076192</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1347,11 +1350,11 @@
       </c>
       <c r="I13" s="6" t="n">
         <f aca="false">IF($A13="","",IF($A13=Paramètres!$B$6,SUM($E$13:$E$22),IF($A13=Paramètres!$B$7,SUM($F$13:$F$22),0)))</f>
-        <v>1404.28586025397</v>
+        <v>1424.28586025397</v>
       </c>
       <c r="J13" s="6" t="n">
         <f aca="false">IF($A13="","",G13+D13+H13+IF(B13="Joint",E13+F13,0)-C13-I13)</f>
-        <v>995.714139746026</v>
+        <v>975.714139746026</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1389,11 +1392,11 @@
       </c>
       <c r="I14" s="6" t="n">
         <f aca="false">IF($A14="","",IF($A14=Paramètres!$B$6,SUM($E$13:$E$22),IF($A14=Paramètres!$B$7,SUM($F$13:$F$22),0)))</f>
-        <v>1199.71413974603</v>
+        <v>1219.71413974603</v>
       </c>
       <c r="J14" s="6" t="n">
         <f aca="false">IF($A14="","",G14+D14+H14+IF(B14="Joint",E14+F14,0)-C14-I14)</f>
-        <v>672.285860253974</v>
+        <v>652.285860253974</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1491,7 +1494,7 @@
       </c>
       <c r="C17" s="6" t="n">
         <f aca="false">IF($A17="","",SUMIFS(Charges!$F$5:$F$54,Charges!$H$5:$H$54,$A17))</f>
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="D17" s="6" t="n">
         <f aca="false">IF($A17="","",SUMIFS(Revenus!$F$5:$F$24,Revenus!$G$5:$G$24,$A17,Revenus!$B$5:$B$24,"&lt;&gt;Salaire"))</f>
@@ -1499,11 +1502,11 @@
       </c>
       <c r="E17" s="11" t="n">
         <f aca="false">IF($A17="","",IF($B17="Joint",IF($C17=0,0,($C17-$D17)*SUMIFS(Charges!$M$5:$M$54,Charges!$H$5:$H$54,$A17)/$C17),0))</f>
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="F17" s="11" t="n">
         <f aca="false">IF($A17="","",IF($B17="Joint",IF($C17=0,0,($C17-$D17)*SUMIFS(Charges!$N$5:$N$54,Charges!$H$5:$H$54,$A17)/$C17),0))</f>
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="G17" s="6" t="n">
         <f aca="false">IF($A17="","",SUMIFS(Revenus!$F$5:$F$24,Revenus!$G$5:$G$24,$A17,Revenus!$B$5:$B$24,"Salaire"))</f>
@@ -1739,7 +1742,7 @@
       <c r="B23" s="8"/>
       <c r="C23" s="9" t="n">
         <f aca="false">SUM(C13:C22)</f>
-        <v>2862</v>
+        <v>2902</v>
       </c>
       <c r="D23" s="9" t="n">
         <f aca="false">SUM(D13:D22)</f>
@@ -1747,11 +1750,11 @@
       </c>
       <c r="E23" s="9" t="n">
         <f aca="false">SUM(E13:E22)</f>
-        <v>1404.28586025397</v>
+        <v>1424.28586025397</v>
       </c>
       <c r="F23" s="9" t="n">
         <f aca="false">SUM(F13:F22)</f>
-        <v>1199.71413974603</v>
+        <v>1219.71413974603</v>
       </c>
       <c r="G23" s="9" t="n">
         <f aca="false">SUM(G13:G22)</f>
@@ -1763,11 +1766,11 @@
       </c>
       <c r="I23" s="9" t="n">
         <f aca="false">SUM(I13:I22)</f>
-        <v>2604</v>
+        <v>2644</v>
       </c>
       <c r="J23" s="9" t="n">
         <f aca="false">SUM(J13:J22)</f>
-        <v>1947</v>
+        <v>1907</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1790,7 +1793,7 @@
       </c>
       <c r="C28" s="7" t="n">
         <f aca="false">IF($B$30=0,0,B28/$B$30)</f>
-        <v>0.604938271604938</v>
+        <v>0.596600045945325</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1799,11 +1802,11 @@
       </c>
       <c r="B29" s="6" t="n">
         <f aca="false">SUMIFS(Charges!$F$5:$F$54,Charges!$C$5:$C$54,"Variable")</f>
-        <v>1130.66666666667</v>
+        <v>1170.66666666667</v>
       </c>
       <c r="C29" s="7" t="n">
         <f aca="false">IF($B$30=0,0,B29/$B$30)</f>
-        <v>0.395061728395062</v>
+        <v>0.403399954054675</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1812,7 +1815,7 @@
       </c>
       <c r="B30" s="9" t="n">
         <f aca="false">B28+B29</f>
-        <v>2862</v>
+        <v>2902</v>
       </c>
       <c r="C30" s="10" t="n">
         <f aca="false">C28+C29</f>
@@ -2482,20 +2485,20 @@
         <v>106</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>28</v>
+        <v>105</v>
       </c>
       <c r="D9" s="13" t="s">
         <v>36</v>
       </c>
       <c r="E9" s="18" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="F9" s="6" t="n">
         <f aca="false">IF(A9="","",IFERROR(E9/INDEX(Paramètres!$E$4:$E$7,MATCH(D9,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="G9" s="13" t="s">
         <v>98</v>
@@ -2505,7 +2508,7 @@
       </c>
       <c r="I9" s="13"/>
       <c r="J9" s="13" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="K9" s="13" t="s">
         <v>101</v>
@@ -2516,181 +2519,179 @@
       </c>
       <c r="M9" s="6" t="n">
         <f aca="false">IF(A9="","",F9*L9)</f>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="N9" s="6" t="n">
         <f aca="false">IF(A9="","",F9-M9)</f>
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="B10" s="13" t="s">
         <v>108</v>
-      </c>
-      <c r="B10" s="13" t="s">
-        <v>109</v>
       </c>
       <c r="C10" s="13" t="s">
         <v>28</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E10" s="18" t="n">
-        <v>210</v>
+        <v>30</v>
       </c>
       <c r="F10" s="6" t="n">
         <f aca="false">IF(A10="","",IFERROR(E10/INDEX(Paramètres!$E$4:$E$7,MATCH(D10,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="G10" s="13" t="s">
         <v>98</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I10" s="13"/>
       <c r="J10" s="13" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="K10" s="13" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="L10" s="7" t="n">
         <f aca="false">IF(A10="","",IF(K10="50/50",0.5,IF(K10="Prorata salaires",Paramètres!$B$9,IF(K10="Personne 1 seul",1,IF(K10="Personne 2 seul",0,0.5)))))</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="M10" s="6" t="n">
         <f aca="false">IF(A10="","",F10*L10)</f>
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="N10" s="6" t="n">
         <f aca="false">IF(A10="","",F10-M10)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C11" s="13" t="s">
         <v>28</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E11" s="18" t="n">
-        <v>28</v>
+        <v>210</v>
       </c>
       <c r="F11" s="6" t="n">
         <f aca="false">IF(A11="","",IFERROR(E11/INDEX(Paramètres!$E$4:$E$7,MATCH(D11,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="G11" s="13" t="s">
         <v>98</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="I11" s="13"/>
       <c r="J11" s="13" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="K11" s="13" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="L11" s="7" t="n">
         <f aca="false">IF(A11="","",IF(K11="50/50",0.5,IF(K11="Prorata salaires",Paramètres!$B$9,IF(K11="Personne 1 seul",1,IF(K11="Personne 2 seul",0,0.5)))))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M11" s="6" t="n">
         <f aca="false">IF(A11="","",F11*L11)</f>
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="N11" s="6" t="n">
         <f aca="false">IF(A11="","",F11-M11)</f>
-        <v>28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>105</v>
+        <v>28</v>
       </c>
       <c r="D12" s="13" t="s">
         <v>36</v>
       </c>
       <c r="E12" s="18" t="n">
-        <v>600</v>
+        <v>28</v>
       </c>
       <c r="F12" s="6" t="n">
         <f aca="false">IF(A12="","",IFERROR(E12/INDEX(Paramètres!$E$4:$E$7,MATCH(D12,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v>600</v>
+        <v>28</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>74</v>
+        <v>44</v>
       </c>
       <c r="I12" s="13"/>
-      <c r="J12" s="13"/>
+      <c r="J12" s="13" t="n">
+        <v>8</v>
+      </c>
       <c r="K12" s="13" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="L12" s="7" t="n">
         <f aca="false">IF(A12="","",IF(K12="50/50",0.5,IF(K12="Prorata salaires",Paramètres!$B$9,IF(K12="Personne 1 seul",1,IF(K12="Personne 2 seul",0,0.5)))))</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="M12" s="6" t="n">
         <f aca="false">IF(A12="","",F12*L12)</f>
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="N12" s="6" t="n">
         <f aca="false">IF(A12="","",F12-M12)</f>
-        <v>300</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>28</v>
+        <v>105</v>
       </c>
       <c r="D13" s="13" t="s">
         <v>36</v>
       </c>
       <c r="E13" s="18" t="n">
-        <v>150</v>
+        <v>600</v>
       </c>
       <c r="F13" s="6" t="n">
         <f aca="false">IF(A13="","",IFERROR(E13/INDEX(Paramètres!$E$4:$E$7,MATCH(D13,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v>150</v>
+        <v>600</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H13" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="I13" s="13" t="s">
-        <v>78</v>
-      </c>
-      <c r="J13" s="13" t="n">
-        <v>3</v>
-      </c>
+      <c r="I13" s="13"/>
+      <c r="J13" s="13"/>
       <c r="K13" s="13" t="s">
         <v>101</v>
       </c>
@@ -2700,44 +2701,44 @@
       </c>
       <c r="M13" s="6" t="n">
         <f aca="false">IF(A13="","",F13*L13)</f>
-        <v>75</v>
+        <v>300</v>
       </c>
       <c r="N13" s="6" t="n">
         <f aca="false">IF(A13="","",F13-M13)</f>
-        <v>75</v>
+        <v>300</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>119</v>
+        <v>79</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>105</v>
+        <v>28</v>
       </c>
       <c r="D14" s="13" t="s">
         <v>36</v>
       </c>
       <c r="E14" s="18" t="n">
-        <v>90</v>
+        <v>150</v>
       </c>
       <c r="F14" s="6" t="n">
         <f aca="false">IF(A14="","",IFERROR(E14/INDEX(Paramètres!$E$4:$E$7,MATCH(D14,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v>90</v>
+        <v>150</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H14" s="13" t="s">
         <v>74</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>120</v>
+        <v>78</v>
       </c>
       <c r="J14" s="13" t="n">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="K14" s="13" t="s">
         <v>101</v>
@@ -2748,41 +2749,45 @@
       </c>
       <c r="M14" s="6" t="n">
         <f aca="false">IF(A14="","",F14*L14)</f>
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="N14" s="6" t="n">
         <f aca="false">IF(A14="","",F14-M14)</f>
-        <v>45</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C15" s="13" t="s">
         <v>105</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="E15" s="18" t="n">
-        <v>600</v>
+        <v>90</v>
       </c>
       <c r="F15" s="6" t="n">
         <f aca="false">IF(A15="","",IFERROR(E15/INDEX(Paramètres!$E$4:$E$7,MATCH(D15,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="H15" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="I15" s="13"/>
-      <c r="J15" s="13"/>
+      <c r="I15" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="J15" s="13" t="n">
+        <v>28</v>
+      </c>
       <c r="K15" s="13" t="s">
         <v>101</v>
       </c>
@@ -2792,11 +2797,11 @@
       </c>
       <c r="M15" s="6" t="n">
         <f aca="false">IF(A15="","",F15*L15)</f>
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="N15" s="6" t="n">
         <f aca="false">IF(A15="","",F15-M15)</f>
-        <v>25</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2804,23 +2809,23 @@
         <v>122</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C16" s="13" t="s">
         <v>105</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="E16" s="18" t="n">
-        <v>30</v>
+        <v>600</v>
       </c>
       <c r="F16" s="6" t="n">
         <f aca="false">IF(A16="","",IFERROR(E16/INDEX(Paramètres!$E$4:$E$7,MATCH(D16,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="H16" s="13" t="s">
         <v>74</v>
@@ -2836,35 +2841,35 @@
       </c>
       <c r="M16" s="6" t="n">
         <f aca="false">IF(A16="","",F16*L16)</f>
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="N16" s="6" t="n">
         <f aca="false">IF(A16="","",F16-M16)</f>
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C17" s="13" t="s">
         <v>105</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="E17" s="18" t="n">
-        <v>500</v>
+        <v>30</v>
       </c>
       <c r="F17" s="6" t="n">
         <f aca="false">IF(A17="","",IFERROR(E17/INDEX(Paramètres!$E$4:$E$7,MATCH(D17,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v>41.6666666666667</v>
+        <v>30</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="H17" s="13" t="s">
         <v>74</v>
@@ -2880,46 +2885,41 @@
       </c>
       <c r="M17" s="6" t="n">
         <f aca="false">IF(A17="","",F17*L17)</f>
-        <v>20.8333333333333</v>
+        <v>15</v>
       </c>
       <c r="N17" s="6" t="n">
         <f aca="false">IF(A17="","",F17-M17)</f>
-        <v>20.8333333333333</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="B18" s="13" t="s">
         <v>127</v>
-      </c>
-      <c r="B18" s="13" t="s">
-        <v>128</v>
       </c>
       <c r="C18" s="13" t="s">
         <v>105</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="E18" s="21" t="n">
-        <f aca="false">Paramètres!$B$22*SUMIFS(Revenus!$F$5:$F$24,Revenus!$B$5:$B$24,"Salaire")</f>
-        <v>129</v>
+        <v>45</v>
+      </c>
+      <c r="E18" s="18" t="n">
+        <v>500</v>
       </c>
       <c r="F18" s="6" t="n">
         <f aca="false">IF(A18="","",IFERROR(E18/INDEX(Paramètres!$E$4:$E$7,MATCH(D18,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v>129</v>
+        <v>41.6666666666667</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H18" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="I18" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="J18" s="13" t="n">
-        <v>3</v>
-      </c>
+      <c r="I18" s="13"/>
+      <c r="J18" s="13"/>
       <c r="K18" s="13" t="s">
         <v>101</v>
       </c>
@@ -2929,42 +2929,45 @@
       </c>
       <c r="M18" s="6" t="n">
         <f aca="false">IF(A18="","",F18*L18)</f>
-        <v>64.5</v>
+        <v>20.8333333333333</v>
       </c>
       <c r="N18" s="6" t="n">
         <f aca="false">IF(A18="","",F18-M18)</f>
-        <v>64.5</v>
+        <v>20.8333333333333</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="B19" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="B19" s="13" t="s">
-        <v>130</v>
-      </c>
       <c r="C19" s="13" t="s">
-        <v>28</v>
+        <v>105</v>
       </c>
       <c r="D19" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="E19" s="18" t="n">
-        <v>120</v>
+      <c r="E19" s="21" t="n">
+        <f aca="false">Paramètres!$B$22*SUMIFS(Revenus!$F$5:$F$24,Revenus!$B$5:$B$24,"Salaire")</f>
+        <v>129</v>
       </c>
       <c r="F19" s="6" t="n">
         <f aca="false">IF(A19="","",IFERROR(E19/INDEX(Paramètres!$E$4:$E$7,MATCH(D19,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="H19" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="I19" s="13"/>
+      <c r="I19" s="13" t="s">
+        <v>81</v>
+      </c>
       <c r="J19" s="13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K19" s="13" t="s">
         <v>101</v>
@@ -2975,19 +2978,19 @@
       </c>
       <c r="M19" s="6" t="n">
         <f aca="false">IF(A19="","",F19*L19)</f>
-        <v>60</v>
+        <v>64.5</v>
       </c>
       <c r="N19" s="6" t="n">
         <f aca="false">IF(A19="","",F19-M19)</f>
-        <v>60</v>
+        <v>64.5</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="C20" s="13" t="s">
         <v>28</v>
@@ -2996,14 +2999,14 @@
         <v>36</v>
       </c>
       <c r="E20" s="18" t="n">
-        <v>30</v>
+        <v>120</v>
       </c>
       <c r="F20" s="6" t="n">
         <f aca="false">IF(A20="","",IFERROR(E20/INDEX(Paramètres!$E$4:$E$7,MATCH(D20,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v>30</v>
+        <v>120</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H20" s="13" t="s">
         <v>74</v>
@@ -3021,11 +3024,11 @@
       </c>
       <c r="M20" s="6" t="n">
         <f aca="false">IF(A20="","",F20*L20)</f>
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="N20" s="6" t="n">
         <f aca="false">IF(A20="","",F20-M20)</f>
-        <v>15</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3033,29 +3036,31 @@
         <v>133</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>105</v>
+        <v>28</v>
       </c>
       <c r="D21" s="13" t="s">
         <v>36</v>
       </c>
       <c r="E21" s="18" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F21" s="6" t="n">
         <f aca="false">IF(A21="","",IFERROR(E21/INDEX(Paramètres!$E$4:$E$7,MATCH(D21,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H21" s="13" t="s">
         <v>74</v>
       </c>
       <c r="I21" s="13"/>
-      <c r="J21" s="13"/>
+      <c r="J21" s="13" t="n">
+        <v>1</v>
+      </c>
       <c r="K21" s="13" t="s">
         <v>101</v>
       </c>
@@ -3065,39 +3070,55 @@
       </c>
       <c r="M21" s="6" t="n">
         <f aca="false">IF(A21="","",F21*L21)</f>
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="N21" s="6" t="n">
         <f aca="false">IF(A21="","",F21-M21)</f>
-        <v>30</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="13"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="18"/>
-      <c r="F22" s="6" t="str">
+      <c r="A22" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E22" s="18" t="n">
+        <v>60</v>
+      </c>
+      <c r="F22" s="6" t="n">
         <f aca="false">IF(A22="","",IFERROR(E22/INDEX(Paramètres!$E$4:$E$7,MATCH(D22,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v/>
-      </c>
-      <c r="G22" s="13"/>
-      <c r="H22" s="13"/>
+        <v>60</v>
+      </c>
+      <c r="G22" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="H22" s="13" t="s">
+        <v>74</v>
+      </c>
       <c r="I22" s="13"/>
       <c r="J22" s="13"/>
-      <c r="K22" s="13"/>
-      <c r="L22" s="7" t="str">
+      <c r="K22" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="L22" s="7" t="n">
         <f aca="false">IF(A22="","",IF(K22="50/50",0.5,IF(K22="Prorata salaires",Paramètres!$B$9,IF(K22="Personne 1 seul",1,IF(K22="Personne 2 seul",0,0.5)))))</f>
-        <v/>
-      </c>
-      <c r="M22" s="6" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="M22" s="6" t="n">
         <f aca="false">IF(A22="","",F22*L22)</f>
-        <v/>
-      </c>
-      <c r="N22" s="6" t="str">
+        <v>30</v>
+      </c>
+      <c r="N22" s="6" t="n">
         <f aca="false">IF(A22="","",F22-M22)</f>
-        <v/>
+        <v>30</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3998,19 +4019,19 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="22" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F55" s="9" t="n">
         <f aca="false">SUM(F5:F54)</f>
-        <v>2862</v>
+        <v>2902</v>
       </c>
       <c r="M55" s="9" t="n">
         <f aca="false">SUM(M5:M54)</f>
-        <v>1525.15891472868</v>
+        <v>1545.15891472868</v>
       </c>
       <c r="N55" s="9" t="n">
         <f aca="false">SUM(N5:N54)</f>
-        <v>1336.84108527132</v>
+        <v>1356.84108527132</v>
       </c>
     </row>
   </sheetData>
@@ -4065,12 +4086,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4093,7 +4114,7 @@
         <v>89</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>93</v>
@@ -4101,10 +4122,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>35</v>
@@ -4128,10 +4149,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="B6" s="13" t="s">
         <v>140</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>139</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>38</v>
@@ -4155,13 +4176,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D7" s="18" t="n">
         <v>140</v>
@@ -4182,13 +4203,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="C8" s="13" t="s">
         <v>144</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>143</v>
       </c>
       <c r="D8" s="18" t="n">
         <v>270</v>
@@ -4417,7 +4438,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="22" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F25" s="9" t="n">
         <f aca="false">SUM(F5:F24)</f>
@@ -4468,12 +4489,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4507,13 +4528,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B5" s="13" t="s">
         <v>35</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>36</v>
@@ -4537,13 +4558,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>35</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D6" s="13" t="s">
         <v>39</v>
@@ -4556,7 +4577,7 @@
         <v>40</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H6" s="13" t="s">
         <v>41</v>
@@ -4565,13 +4586,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B7" s="13" t="s">
         <v>35</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D7" s="13" t="s">
         <v>36</v>
@@ -5113,7 +5134,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="22" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F45" s="9" t="n">
         <f aca="false">SUM(F5:F44)</f>
@@ -5122,20 +5143,20 @@
     </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G44" type="list">
-      <formula1>"Prélèvement,Carte,Chèque,Espèces,Virement"</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D44" type="list">
+      <formula1>"Mensuelle,Trimestrielle,Semestrielle,Annuelle"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H44" type="list">
       <formula1>Comptes!$A$5:$A$14</formula1>
       <formula2>0</formula2>
     </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G44" type="list">
+      <formula1>"Prélèvement,Carte,Chèque,Espèces,Virement"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B44" type="list">
       <formula1>Paramètres!$B$4:$B$5</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D44" type="list">
-      <formula1>"Mensuelle,Trimestrielle,Semestrielle,Annuelle"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -5165,17 +5186,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="23" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B4" s="6" t="n">
         <f aca="false">SUMIFS(Charges!$F$5:$F$54,Charges!$B$5:$B$54,"Imprévus")</f>
@@ -5184,7 +5205,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B5" s="24" t="n">
         <v>46266</v>
@@ -5192,7 +5213,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>0</v>
@@ -5200,7 +5221,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B7" s="25" t="n">
         <f aca="true">IF(B5="",0,MAX(0,(YEAR(TODAY())-YEAR(B5))*12+MONTH(TODAY())-MONTH(B5)+1))</f>
@@ -5209,7 +5230,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B8" s="6" t="n">
         <f aca="false">B6+B4*B7</f>
@@ -5218,7 +5239,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">SUM(C13:C62)</f>
@@ -5227,7 +5248,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">B8-B9</f>
@@ -5236,21 +5257,21 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>85</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5258,7 +5279,7 @@
         <v>46285</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C13" s="18" t="n">
         <v>220</v>
@@ -5272,7 +5293,7 @@
         <v>46300</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C14" s="18" t="n">
         <v>85</v>

</xml_diff>

<commit_message>
Ajout de CLAUDE.md, du versionnement du modèle (1.0.0) et du mécanisme de migration
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KqkJNWVZSWN9upSPoUaH5h
</commit_message>
<xml_diff>
--- a/suivi_comptes_example.xlsx
+++ b/suivi_comptes_example.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="170">
   <si>
     <t xml:space="preserve">Synthèse mensuelle</t>
   </si>
@@ -212,6 +212,15 @@
   </si>
   <si>
     <t xml:space="preserve">Alimente la ligne « Provision imprévus » de l'onglet Charges (réparties 50/50, sur le compte joint indiqué).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Version du modèle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voir MIGRATION.md pour migrer un fichier d'une version à l'autre.</t>
   </si>
   <si>
     <t xml:space="preserve">Comptes bancaires</t>
@@ -1838,7 +1847,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
@@ -2024,6 +2033,19 @@
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
         <v>61</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -2063,26 +2085,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>18</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2090,13 +2112,13 @@
         <v>41</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>35</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2104,83 +2126,83 @@
         <v>44</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>38</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="B8" s="13" t="s">
-        <v>71</v>
-      </c>
       <c r="C8" s="13" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2242,50 +2264,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="M4" s="4" t="str">
         <f aca="false">"Part "&amp;Paramètres!$B$4&amp;" (€/mois)"</f>
@@ -2298,10 +2320,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>28</v>
@@ -2317,17 +2339,17 @@
         <v>1150</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I5" s="13"/>
       <c r="J5" s="13" t="n">
         <v>5</v>
       </c>
       <c r="K5" s="13" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="L5" s="7" t="n">
         <f aca="false">IF(A5="","",IF(K5="50/50",0.5,IF(K5="Prorata salaires",Paramètres!$B$9,IF(K5="Personne 1 seul",1,IF(K5="Personne 2 seul",0,0.5)))))</f>
@@ -2344,10 +2366,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" s="13" t="s">
         <v>100</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>97</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>28</v>
@@ -2363,17 +2385,17 @@
         <v>45</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="H6" s="13" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I6" s="13"/>
       <c r="J6" s="13" t="n">
         <v>5</v>
       </c>
       <c r="K6" s="13" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="L6" s="7" t="n">
         <f aca="false">IF(A6="","",IF(K6="50/50",0.5,IF(K6="Prorata salaires",Paramètres!$B$9,IF(K6="Personne 1 seul",1,IF(K6="Personne 2 seul",0,0.5)))))</f>
@@ -2390,10 +2412,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C7" s="13" t="s">
         <v>28</v>
@@ -2409,17 +2431,17 @@
         <v>108.333333333333</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="H7" s="13" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I7" s="13"/>
       <c r="J7" s="13" t="n">
         <v>15</v>
       </c>
       <c r="K7" s="13" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="L7" s="7" t="n">
         <f aca="false">IF(A7="","",IF(K7="50/50",0.5,IF(K7="Prorata salaires",Paramètres!$B$9,IF(K7="Personne 1 seul",1,IF(K7="Personne 2 seul",0,0.5)))))</f>
@@ -2436,13 +2458,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D8" s="13" t="s">
         <v>36</v>
@@ -2455,17 +2477,17 @@
         <v>130</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="H8" s="13" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I8" s="13"/>
       <c r="J8" s="13" t="n">
         <v>12</v>
       </c>
       <c r="K8" s="13" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="L8" s="7" t="n">
         <f aca="false">IF(A8="","",IF(K8="50/50",0.5,IF(K8="Prorata salaires",Paramètres!$B$9,IF(K8="Personne 1 seul",1,IF(K8="Personne 2 seul",0,0.5)))))</f>
@@ -2482,13 +2504,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D9" s="13" t="s">
         <v>36</v>
@@ -2501,17 +2523,17 @@
         <v>40</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I9" s="13"/>
       <c r="J9" s="13" t="n">
         <v>14</v>
       </c>
       <c r="K9" s="13" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="L9" s="7" t="n">
         <f aca="false">IF(A9="","",IF(K9="50/50",0.5,IF(K9="Prorata salaires",Paramètres!$B$9,IF(K9="Personne 1 seul",1,IF(K9="Personne 2 seul",0,0.5)))))</f>
@@ -2528,10 +2550,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C10" s="13" t="s">
         <v>28</v>
@@ -2547,17 +2569,17 @@
         <v>30</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I10" s="13"/>
       <c r="J10" s="13" t="n">
         <v>10</v>
       </c>
       <c r="K10" s="13" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="L10" s="7" t="n">
         <f aca="false">IF(A10="","",IF(K10="50/50",0.5,IF(K10="Prorata salaires",Paramètres!$B$9,IF(K10="Personne 1 seul",1,IF(K10="Personne 2 seul",0,0.5)))))</f>
@@ -2574,10 +2596,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C11" s="13" t="s">
         <v>28</v>
@@ -2593,17 +2615,17 @@
         <v>70</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I11" s="13"/>
       <c r="J11" s="13" t="n">
         <v>1</v>
       </c>
       <c r="K11" s="13" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="L11" s="7" t="n">
         <f aca="false">IF(A11="","",IF(K11="50/50",0.5,IF(K11="Prorata salaires",Paramètres!$B$9,IF(K11="Personne 1 seul",1,IF(K11="Personne 2 seul",0,0.5)))))</f>
@@ -2620,10 +2642,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>28</v>
@@ -2639,7 +2661,7 @@
         <v>28</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="H12" s="13" t="s">
         <v>44</v>
@@ -2649,7 +2671,7 @@
         <v>8</v>
       </c>
       <c r="K12" s="13" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="L12" s="7" t="n">
         <f aca="false">IF(A12="","",IF(K12="50/50",0.5,IF(K12="Prorata salaires",Paramètres!$B$9,IF(K12="Personne 1 seul",1,IF(K12="Personne 2 seul",0,0.5)))))</f>
@@ -2666,13 +2688,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D13" s="13" t="s">
         <v>36</v>
@@ -2685,15 +2707,15 @@
         <v>600</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I13" s="13"/>
       <c r="J13" s="13"/>
       <c r="K13" s="13" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="L13" s="7" t="n">
         <f aca="false">IF(A13="","",IF(K13="50/50",0.5,IF(K13="Prorata salaires",Paramètres!$B$9,IF(K13="Personne 1 seul",1,IF(K13="Personne 2 seul",0,0.5)))))</f>
@@ -2710,10 +2732,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C14" s="13" t="s">
         <v>28</v>
@@ -2729,19 +2751,19 @@
         <v>150</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J14" s="13" t="n">
         <v>3</v>
       </c>
       <c r="K14" s="13" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="L14" s="7" t="n">
         <f aca="false">IF(A14="","",IF(K14="50/50",0.5,IF(K14="Prorata salaires",Paramètres!$B$9,IF(K14="Personne 1 seul",1,IF(K14="Personne 2 seul",0,0.5)))))</f>
@@ -2758,13 +2780,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D15" s="13" t="s">
         <v>36</v>
@@ -2777,19 +2799,19 @@
         <v>90</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="J15" s="13" t="n">
         <v>28</v>
       </c>
       <c r="K15" s="13" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="L15" s="7" t="n">
         <f aca="false">IF(A15="","",IF(K15="50/50",0.5,IF(K15="Prorata salaires",Paramètres!$B$9,IF(K15="Personne 1 seul",1,IF(K15="Personne 2 seul",0,0.5)))))</f>
@@ -2806,13 +2828,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D16" s="13" t="s">
         <v>45</v>
@@ -2825,15 +2847,15 @@
         <v>50</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I16" s="13"/>
       <c r="J16" s="13"/>
       <c r="K16" s="13" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="L16" s="7" t="n">
         <f aca="false">IF(A16="","",IF(K16="50/50",0.5,IF(K16="Prorata salaires",Paramètres!$B$9,IF(K16="Personne 1 seul",1,IF(K16="Personne 2 seul",0,0.5)))))</f>
@@ -2850,13 +2872,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D17" s="13" t="s">
         <v>36</v>
@@ -2869,15 +2891,15 @@
         <v>30</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I17" s="13"/>
       <c r="J17" s="13"/>
       <c r="K17" s="13" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="L17" s="7" t="n">
         <f aca="false">IF(A17="","",IF(K17="50/50",0.5,IF(K17="Prorata salaires",Paramètres!$B$9,IF(K17="Personne 1 seul",1,IF(K17="Personne 2 seul",0,0.5)))))</f>
@@ -2894,13 +2916,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D18" s="13" t="s">
         <v>45</v>
@@ -2913,15 +2935,15 @@
         <v>41.6666666666667</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I18" s="13"/>
       <c r="J18" s="13"/>
       <c r="K18" s="13" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="L18" s="7" t="n">
         <f aca="false">IF(A18="","",IF(K18="50/50",0.5,IF(K18="Prorata salaires",Paramètres!$B$9,IF(K18="Personne 1 seul",1,IF(K18="Personne 2 seul",0,0.5)))))</f>
@@ -2938,13 +2960,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D19" s="13" t="s">
         <v>36</v>
@@ -2958,19 +2980,19 @@
         <v>129</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I19" s="13" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="J19" s="13" t="n">
         <v>3</v>
       </c>
       <c r="K19" s="13" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="L19" s="7" t="n">
         <f aca="false">IF(A19="","",IF(K19="50/50",0.5,IF(K19="Prorata salaires",Paramètres!$B$9,IF(K19="Personne 1 seul",1,IF(K19="Personne 2 seul",0,0.5)))))</f>
@@ -2987,10 +3009,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C20" s="13" t="s">
         <v>28</v>
@@ -3006,17 +3028,17 @@
         <v>120</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I20" s="13"/>
       <c r="J20" s="13" t="n">
         <v>1</v>
       </c>
       <c r="K20" s="13" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="L20" s="7" t="n">
         <f aca="false">IF(A20="","",IF(K20="50/50",0.5,IF(K20="Prorata salaires",Paramètres!$B$9,IF(K20="Personne 1 seul",1,IF(K20="Personne 2 seul",0,0.5)))))</f>
@@ -3033,10 +3055,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C21" s="13" t="s">
         <v>28</v>
@@ -3052,17 +3074,17 @@
         <v>30</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I21" s="13"/>
       <c r="J21" s="13" t="n">
         <v>1</v>
       </c>
       <c r="K21" s="13" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="L21" s="7" t="n">
         <f aca="false">IF(A21="","",IF(K21="50/50",0.5,IF(K21="Prorata salaires",Paramètres!$B$9,IF(K21="Personne 1 seul",1,IF(K21="Personne 2 seul",0,0.5)))))</f>
@@ -3079,13 +3101,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D22" s="13" t="s">
         <v>36</v>
@@ -3098,15 +3120,15 @@
         <v>60</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I22" s="13"/>
       <c r="J22" s="13"/>
       <c r="K22" s="13" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="L22" s="7" t="n">
         <f aca="false">IF(A22="","",IF(K22="50/50",0.5,IF(K22="Prorata salaires",Paramètres!$B$9,IF(K22="Personne 1 seul",1,IF(K22="Personne 2 seul",0,0.5)))))</f>
@@ -4019,7 +4041,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="22" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F55" s="9" t="n">
         <f aca="false">SUM(F5:F54)</f>
@@ -4036,20 +4058,20 @@
     </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C5:C54" type="list">
-      <formula1>"Fixe,Variable"</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H54" type="list">
+      <formula1>Comptes!$A$5:$A$14</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D54" type="list">
       <formula1>"Mensuelle,Trimestrielle,Semestrielle,Annuelle"</formula1>
       <formula2>0</formula2>
     </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C5:C54" type="list">
+      <formula1>"Fixe,Variable"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G54" type="list">
       <formula1>"Prélèvement,Virement,Carte,Chèque,Espèces"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H54" type="list">
-      <formula1>Comptes!$A$5:$A$14</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K5:K54" type="list">
@@ -4086,17 +4108,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>18</v>
@@ -4105,27 +4127,27 @@
         <v>3</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>32</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>35</v>
@@ -4149,10 +4171,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>38</v>
@@ -4176,13 +4198,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D7" s="18" t="n">
         <v>140</v>
@@ -4195,7 +4217,7 @@
         <v>140</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="H7" s="13" t="n">
         <v>5</v>
@@ -4203,13 +4225,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D8" s="18" t="n">
         <v>270</v>
@@ -4222,7 +4244,7 @@
         <v>90</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="H8" s="13" t="n">
         <v>5</v>
@@ -4438,7 +4460,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="22" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F25" s="9" t="n">
         <f aca="false">SUM(F5:F24)</f>
@@ -4489,52 +4511,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B5" s="13" t="s">
         <v>35</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>36</v>
@@ -4547,7 +4569,7 @@
         <v>35</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="H5" s="13" t="s">
         <v>41</v>
@@ -4558,13 +4580,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>35</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D6" s="13" t="s">
         <v>39</v>
@@ -4577,7 +4599,7 @@
         <v>40</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="H6" s="13" t="s">
         <v>41</v>
@@ -4586,13 +4608,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B7" s="13" t="s">
         <v>35</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D7" s="13" t="s">
         <v>36</v>
@@ -4605,7 +4627,7 @@
         <v>11</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="H7" s="13" t="s">
         <v>41</v>
@@ -5134,7 +5156,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="22" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F45" s="9" t="n">
         <f aca="false">SUM(F5:F44)</f>
@@ -5143,20 +5165,20 @@
     </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D44" type="list">
-      <formula1>"Mensuelle,Trimestrielle,Semestrielle,Annuelle"</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G44" type="list">
+      <formula1>"Prélèvement,Carte,Chèque,Espèces,Virement"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H44" type="list">
       <formula1>Comptes!$A$5:$A$14</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G44" type="list">
-      <formula1>"Prélèvement,Carte,Chèque,Espèces,Virement"</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B44" type="list">
+      <formula1>Paramètres!$B$4:$B$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B44" type="list">
-      <formula1>Paramètres!$B$4:$B$5</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D44" type="list">
+      <formula1>"Mensuelle,Trimestrielle,Semestrielle,Annuelle"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -5186,17 +5208,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="23" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B4" s="6" t="n">
         <f aca="false">SUMIFS(Charges!$F$5:$F$54,Charges!$B$5:$B$54,"Imprévus")</f>
@@ -5205,7 +5227,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B5" s="24" t="n">
         <v>46266</v>
@@ -5213,7 +5235,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>0</v>
@@ -5221,7 +5243,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B7" s="25" t="n">
         <f aca="true">IF(B5="",0,MAX(0,(YEAR(TODAY())-YEAR(B5))*12+MONTH(TODAY())-MONTH(B5)+1))</f>
@@ -5230,7 +5252,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B8" s="6" t="n">
         <f aca="false">B6+B4*B7</f>
@@ -5239,7 +5261,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">SUM(C13:C62)</f>
@@ -5248,7 +5270,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">B8-B9</f>
@@ -5257,21 +5279,21 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5279,13 +5301,13 @@
         <v>46285</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C13" s="18" t="n">
         <v>220</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5293,13 +5315,13 @@
         <v>46300</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C14" s="18" t="n">
         <v>85</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Exemple d'épargne enfants : un livret par enfant alimenté depuis le compte joint
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KqkJNWVZSWN9upSPoUaH5h
</commit_message>
<xml_diff>
--- a/suivi_comptes_example.xlsx
+++ b/suivi_comptes_example.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="178">
   <si>
     <t xml:space="preserve">Synthèse mensuelle</t>
   </si>
@@ -286,6 +286,24 @@
     <t xml:space="preserve">Provision pour les dépenses imprévues</t>
   </si>
   <si>
+    <t xml:space="preserve">Livret enfant 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enfant 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Épargne de l'enfant 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Livret enfant 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enfant 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Épargne de l'enfant 2</t>
+  </si>
+  <si>
     <t xml:space="preserve">Charges (dépenses récurrentes)</t>
   </si>
   <si>
@@ -425,6 +443,12 @@
   </si>
   <si>
     <t xml:space="preserve">Imprévus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Épargne enfant 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Épargne enfant 2</t>
   </si>
   <si>
     <t xml:space="preserve">Aide à domicile (retrait espèces)</t>
@@ -1154,7 +1178,7 @@
       </c>
       <c r="C5" s="6" t="n">
         <f aca="false">SUM(E$13:E$22)</f>
-        <v>1424.28586025397</v>
+        <v>1474.68520665978</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">IF(Paramètres!$B$6="",0,IFERROR(INDEX($C$13:$C$22,MATCH(Paramètres!$B$6,$A$13:$A$22,0)),0))</f>
@@ -1162,15 +1186,15 @@
       </c>
       <c r="E5" s="6" t="n">
         <f aca="false">C5+D5</f>
-        <v>1424.28586025397</v>
+        <v>1474.68520665978</v>
       </c>
       <c r="F5" s="7" t="n">
         <f aca="false">IF(B5=0,0,E5/B5)</f>
-        <v>0.593452441772489</v>
+        <v>0.614452169441575</v>
       </c>
       <c r="G5" s="6" t="n">
         <f aca="false">IF(Paramètres!$B$6="",0,IFERROR(INDEX($J$13:$J$22,MATCH(Paramètres!$B$6,$A$13:$A$22,0)),0))</f>
-        <v>975.714139746026</v>
+        <v>925.314793340221</v>
       </c>
       <c r="H5" s="6" t="n">
         <f aca="false">IF(Paramètres!B$15="Forfait",Paramètres!B$16,SUMIFS('Charges perso'!$F$5:$F$44,'Charges perso'!$B$5:$B$44,A5))</f>
@@ -1178,15 +1202,15 @@
       </c>
       <c r="I5" s="6" t="n">
         <f aca="false">G5-H5</f>
-        <v>889.714139746026</v>
+        <v>839.314793340221</v>
       </c>
       <c r="J5" s="6" t="n">
         <f aca="false">MAX(0,IF(Paramètres!B$17="Pourcentage",Paramètres!B$18*MAX(0,I5),Paramètres!B$19))</f>
-        <v>266.914241923808</v>
+        <v>251.794438002066</v>
       </c>
       <c r="K5" s="6" t="n">
         <f aca="false">I5-J5</f>
-        <v>622.799897822218</v>
+        <v>587.520355338154</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1200,7 +1224,7 @@
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">SUM(F$13:F$22)</f>
-        <v>1219.71413974603</v>
+        <v>1269.31479334022</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">IF(Paramètres!$B$7="",0,IFERROR(INDEX($C$13:$C$22,MATCH(Paramètres!$B$7,$A$13:$A$22,0)),0))</f>
@@ -1208,15 +1232,15 @@
       </c>
       <c r="E6" s="6" t="n">
         <f aca="false">C6+D6</f>
-        <v>1247.71413974603</v>
+        <v>1297.31479334022</v>
       </c>
       <c r="F6" s="7" t="n">
         <f aca="false">IF(B6=0,0,E6/B6)</f>
-        <v>0.656691652497908</v>
+        <v>0.682797259652748</v>
       </c>
       <c r="G6" s="6" t="n">
         <f aca="false">IF(Paramètres!$B$7="",0,IFERROR(INDEX($J$13:$J$22,MATCH(Paramètres!$B$7,$A$13:$A$22,0)),0))</f>
-        <v>652.285860253974</v>
+        <v>602.685206659779</v>
       </c>
       <c r="H6" s="6" t="n">
         <f aca="false">IF(Paramètres!C$15="Forfait",Paramètres!C$16,SUMIFS('Charges perso'!$F$5:$F$44,'Charges perso'!$B$5:$B$44,A6))</f>
@@ -1224,7 +1248,7 @@
       </c>
       <c r="I6" s="6" t="n">
         <f aca="false">G6-H6</f>
-        <v>302.285860253974</v>
+        <v>252.685206659779</v>
       </c>
       <c r="J6" s="6" t="n">
         <f aca="false">MAX(0,IF(Paramètres!C$17="Pourcentage",Paramètres!C$18*MAX(0,I6),Paramètres!C$19))</f>
@@ -1232,7 +1256,7 @@
       </c>
       <c r="K6" s="6" t="n">
         <f aca="false">I6-J6</f>
-        <v>102.285860253974</v>
+        <v>52.6852066597792</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1245,7 +1269,7 @@
       </c>
       <c r="C7" s="9" t="n">
         <f aca="false">SUM(C5:C6)</f>
-        <v>2644</v>
+        <v>2744</v>
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">SUM(D5:D6)</f>
@@ -1253,15 +1277,15 @@
       </c>
       <c r="E7" s="9" t="n">
         <f aca="false">SUM(E5:E6)</f>
-        <v>2672</v>
+        <v>2772</v>
       </c>
       <c r="F7" s="10" t="n">
         <f aca="false">IF(B7=0,0,E7/B7)</f>
-        <v>0.621395348837209</v>
+        <v>0.644651162790698</v>
       </c>
       <c r="G7" s="9" t="n">
         <f aca="false">SUM(G5:G6)</f>
-        <v>1628</v>
+        <v>1528</v>
       </c>
       <c r="H7" s="9" t="n">
         <f aca="false">SUM(H5:H6)</f>
@@ -1269,15 +1293,15 @@
       </c>
       <c r="I7" s="9" t="n">
         <f aca="false">SUM(I5:I6)</f>
-        <v>1192</v>
+        <v>1092</v>
       </c>
       <c r="J7" s="9" t="n">
         <f aca="false">SUM(J5:J6)</f>
-        <v>466.914241923808</v>
+        <v>451.794438002066</v>
       </c>
       <c r="K7" s="9" t="n">
         <f aca="false">SUM(K5:K6)</f>
-        <v>725.085758076192</v>
+        <v>640.205561997934</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1359,11 +1383,11 @@
       </c>
       <c r="I13" s="6" t="n">
         <f aca="false">IF($A13="","",IF($A13=Paramètres!$B$6,SUM($E$13:$E$22),IF($A13=Paramètres!$B$7,SUM($F$13:$F$22),0)))</f>
-        <v>1424.28586025397</v>
+        <v>1474.68520665978</v>
       </c>
       <c r="J13" s="6" t="n">
         <f aca="false">IF($A13="","",G13+D13+H13+IF(B13="Joint",E13+F13,0)-C13-I13)</f>
-        <v>975.714139746026</v>
+        <v>925.314793340221</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1401,11 +1425,11 @@
       </c>
       <c r="I14" s="6" t="n">
         <f aca="false">IF($A14="","",IF($A14=Paramètres!$B$6,SUM($E$13:$E$22),IF($A14=Paramètres!$B$7,SUM($F$13:$F$22),0)))</f>
-        <v>1219.71413974603</v>
+        <v>1269.31479334022</v>
       </c>
       <c r="J14" s="6" t="n">
         <f aca="false">IF($A14="","",G14+D14+H14+IF(B14="Joint",E14+F14,0)-C14-I14)</f>
-        <v>652.285860253974</v>
+        <v>602.685206659779</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1461,7 +1485,7 @@
       </c>
       <c r="C16" s="6" t="n">
         <f aca="false">IF($A16="","",SUMIFS(Charges!$F$5:$F$54,Charges!$H$5:$H$54,$A16))</f>
-        <v>1370.66666666667</v>
+        <v>1470.66666666667</v>
       </c>
       <c r="D16" s="6" t="n">
         <f aca="false">IF($A16="","",SUMIFS(Revenus!$F$5:$F$24,Revenus!$G$5:$G$24,$A16,Revenus!$B$5:$B$24,"&lt;&gt;Salaire"))</f>
@@ -1469,11 +1493,11 @@
       </c>
       <c r="E16" s="11" t="n">
         <f aca="false">IF($A16="","",IF($B16="Joint",IF($C16=0,0,($C16-$D16)*SUMIFS(Charges!$M$5:$M$54,Charges!$H$5:$H$54,$A16)/$C16),0))</f>
-        <v>599.460278858625</v>
+        <v>649.85962526443</v>
       </c>
       <c r="F16" s="11" t="n">
         <f aca="false">IF($A16="","",IF($B16="Joint",IF($C16=0,0,($C16-$D16)*SUMIFS(Charges!$N$5:$N$54,Charges!$H$5:$H$54,$A16)/$C16),0))</f>
-        <v>541.206387808042</v>
+        <v>590.807041402236</v>
       </c>
       <c r="G16" s="6" t="n">
         <f aca="false">IF($A16="","",SUMIFS(Revenus!$F$5:$F$24,Revenus!$G$5:$G$24,$A16,Revenus!$B$5:$B$24,"Salaire"))</f>
@@ -1621,85 +1645,85 @@
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="str">
         <f aca="false">IF(Comptes!A12="","",Comptes!A12)</f>
-        <v/>
+        <v>Livret enfant 1</v>
       </c>
       <c r="B20" s="5" t="str">
         <f aca="false">IF($A20="","",Comptes!B12)</f>
-        <v/>
-      </c>
-      <c r="C20" s="6" t="str">
+        <v>Épargne</v>
+      </c>
+      <c r="C20" s="6" t="n">
         <f aca="false">IF($A20="","",SUMIFS(Charges!$F$5:$F$54,Charges!$H$5:$H$54,$A20))</f>
-        <v/>
-      </c>
-      <c r="D20" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="D20" s="6" t="n">
         <f aca="false">IF($A20="","",SUMIFS(Revenus!$F$5:$F$24,Revenus!$G$5:$G$24,$A20,Revenus!$B$5:$B$24,"&lt;&gt;Salaire"))</f>
-        <v/>
-      </c>
-      <c r="E20" s="11" t="str">
+        <v>0</v>
+      </c>
+      <c r="E20" s="11" t="n">
         <f aca="false">IF($A20="","",IF($B20="Joint",IF($C20=0,0,($C20-$D20)*SUMIFS(Charges!$M$5:$M$54,Charges!$H$5:$H$54,$A20)/$C20),0))</f>
-        <v/>
-      </c>
-      <c r="F20" s="11" t="str">
+        <v>0</v>
+      </c>
+      <c r="F20" s="11" t="n">
         <f aca="false">IF($A20="","",IF($B20="Joint",IF($C20=0,0,($C20-$D20)*SUMIFS(Charges!$N$5:$N$54,Charges!$H$5:$H$54,$A20)/$C20),0))</f>
-        <v/>
-      </c>
-      <c r="G20" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="G20" s="6" t="n">
         <f aca="false">IF($A20="","",SUMIFS(Revenus!$F$5:$F$24,Revenus!$G$5:$G$24,$A20,Revenus!$B$5:$B$24,"Salaire"))</f>
-        <v/>
-      </c>
-      <c r="H20" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H20" s="6" t="n">
         <f aca="false">IF($A20="","",SUMIFS(Charges!$F$5:$F$54,Charges!$I$5:$I$54,$A20,Charges!$G$5:$G$54,"Virement"))</f>
-        <v/>
-      </c>
-      <c r="I20" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="I20" s="6" t="n">
         <f aca="false">IF($A20="","",IF($A20=Paramètres!$B$6,SUM($E$13:$E$22),IF($A20=Paramètres!$B$7,SUM($F$13:$F$22),0)))</f>
-        <v/>
-      </c>
-      <c r="J20" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="J20" s="6" t="n">
         <f aca="false">IF($A20="","",G20+D20+H20+IF(B20="Joint",E20+F20,0)-C20-I20)</f>
-        <v/>
+        <v>50</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="str">
         <f aca="false">IF(Comptes!A13="","",Comptes!A13)</f>
-        <v/>
+        <v>Livret enfant 2</v>
       </c>
       <c r="B21" s="5" t="str">
         <f aca="false">IF($A21="","",Comptes!B13)</f>
-        <v/>
-      </c>
-      <c r="C21" s="6" t="str">
+        <v>Épargne</v>
+      </c>
+      <c r="C21" s="6" t="n">
         <f aca="false">IF($A21="","",SUMIFS(Charges!$F$5:$F$54,Charges!$H$5:$H$54,$A21))</f>
-        <v/>
-      </c>
-      <c r="D21" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="D21" s="6" t="n">
         <f aca="false">IF($A21="","",SUMIFS(Revenus!$F$5:$F$24,Revenus!$G$5:$G$24,$A21,Revenus!$B$5:$B$24,"&lt;&gt;Salaire"))</f>
-        <v/>
-      </c>
-      <c r="E21" s="11" t="str">
+        <v>0</v>
+      </c>
+      <c r="E21" s="11" t="n">
         <f aca="false">IF($A21="","",IF($B21="Joint",IF($C21=0,0,($C21-$D21)*SUMIFS(Charges!$M$5:$M$54,Charges!$H$5:$H$54,$A21)/$C21),0))</f>
-        <v/>
-      </c>
-      <c r="F21" s="11" t="str">
+        <v>0</v>
+      </c>
+      <c r="F21" s="11" t="n">
         <f aca="false">IF($A21="","",IF($B21="Joint",IF($C21=0,0,($C21-$D21)*SUMIFS(Charges!$N$5:$N$54,Charges!$H$5:$H$54,$A21)/$C21),0))</f>
-        <v/>
-      </c>
-      <c r="G21" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="G21" s="6" t="n">
         <f aca="false">IF($A21="","",SUMIFS(Revenus!$F$5:$F$24,Revenus!$G$5:$G$24,$A21,Revenus!$B$5:$B$24,"Salaire"))</f>
-        <v/>
-      </c>
-      <c r="H21" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H21" s="6" t="n">
         <f aca="false">IF($A21="","",SUMIFS(Charges!$F$5:$F$54,Charges!$I$5:$I$54,$A21,Charges!$G$5:$G$54,"Virement"))</f>
-        <v/>
-      </c>
-      <c r="I21" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="I21" s="6" t="n">
         <f aca="false">IF($A21="","",IF($A21=Paramètres!$B$6,SUM($E$13:$E$22),IF($A21=Paramètres!$B$7,SUM($F$13:$F$22),0)))</f>
-        <v/>
-      </c>
-      <c r="J21" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="J21" s="6" t="n">
         <f aca="false">IF($A21="","",G21+D21+H21+IF(B21="Joint",E21+F21,0)-C21-I21)</f>
-        <v/>
+        <v>50</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1751,7 +1775,7 @@
       <c r="B23" s="8"/>
       <c r="C23" s="9" t="n">
         <f aca="false">SUM(C13:C22)</f>
-        <v>2902</v>
+        <v>3002</v>
       </c>
       <c r="D23" s="9" t="n">
         <f aca="false">SUM(D13:D22)</f>
@@ -1759,11 +1783,11 @@
       </c>
       <c r="E23" s="9" t="n">
         <f aca="false">SUM(E13:E22)</f>
-        <v>1424.28586025397</v>
+        <v>1474.68520665978</v>
       </c>
       <c r="F23" s="9" t="n">
         <f aca="false">SUM(F13:F22)</f>
-        <v>1219.71413974603</v>
+        <v>1269.31479334022</v>
       </c>
       <c r="G23" s="9" t="n">
         <f aca="false">SUM(G13:G22)</f>
@@ -1771,11 +1795,11 @@
       </c>
       <c r="H23" s="9" t="n">
         <f aca="false">SUM(H13:H22)</f>
-        <v>279</v>
+        <v>379</v>
       </c>
       <c r="I23" s="9" t="n">
         <f aca="false">SUM(I13:I22)</f>
-        <v>2644</v>
+        <v>2744</v>
       </c>
       <c r="J23" s="9" t="n">
         <f aca="false">SUM(J13:J22)</f>
@@ -1798,11 +1822,11 @@
       </c>
       <c r="B28" s="6" t="n">
         <f aca="false">SUMIFS(Charges!$F$5:$F$54,Charges!$C$5:$C$54,"Fixe")</f>
-        <v>1731.33333333333</v>
+        <v>1831.33333333333</v>
       </c>
       <c r="C28" s="7" t="n">
         <f aca="false">IF($B$30=0,0,B28/$B$30)</f>
-        <v>0.596600045945325</v>
+        <v>0.610037752609372</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1815,7 +1839,7 @@
       </c>
       <c r="C29" s="7" t="n">
         <f aca="false">IF($B$30=0,0,B29/$B$30)</f>
-        <v>0.403399954054675</v>
+        <v>0.389962247390629</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1824,7 +1848,7 @@
       </c>
       <c r="B30" s="9" t="n">
         <f aca="false">B28+B29</f>
-        <v>2902</v>
+        <v>3002</v>
       </c>
       <c r="C30" s="10" t="n">
         <f aca="false">C28+C29</f>
@@ -2206,16 +2230,32 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13"/>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
+      <c r="A12" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13"/>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
+      <c r="A13" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13"/>
@@ -2264,50 +2304,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="M4" s="4" t="str">
         <f aca="false">"Part "&amp;Paramètres!$B$4&amp;" (€/mois)"</f>
@@ -2320,10 +2360,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>28</v>
@@ -2339,7 +2379,7 @@
         <v>1150</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="H5" s="13" t="s">
         <v>73</v>
@@ -2349,7 +2389,7 @@
         <v>5</v>
       </c>
       <c r="K5" s="13" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="L5" s="7" t="n">
         <f aca="false">IF(A5="","",IF(K5="50/50",0.5,IF(K5="Prorata salaires",Paramètres!$B$9,IF(K5="Personne 1 seul",1,IF(K5="Personne 2 seul",0,0.5)))))</f>
@@ -2366,10 +2406,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>28</v>
@@ -2385,7 +2425,7 @@
         <v>45</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="H6" s="13" t="s">
         <v>73</v>
@@ -2395,7 +2435,7 @@
         <v>5</v>
       </c>
       <c r="K6" s="13" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="L6" s="7" t="n">
         <f aca="false">IF(A6="","",IF(K6="50/50",0.5,IF(K6="Prorata salaires",Paramètres!$B$9,IF(K6="Personne 1 seul",1,IF(K6="Personne 2 seul",0,0.5)))))</f>
@@ -2412,10 +2452,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="C7" s="13" t="s">
         <v>28</v>
@@ -2431,7 +2471,7 @@
         <v>108.333333333333</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="H7" s="13" t="s">
         <v>73</v>
@@ -2441,7 +2481,7 @@
         <v>15</v>
       </c>
       <c r="K7" s="13" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="L7" s="7" t="n">
         <f aca="false">IF(A7="","",IF(K7="50/50",0.5,IF(K7="Prorata salaires",Paramètres!$B$9,IF(K7="Personne 1 seul",1,IF(K7="Personne 2 seul",0,0.5)))))</f>
@@ -2458,13 +2498,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D8" s="13" t="s">
         <v>36</v>
@@ -2477,7 +2517,7 @@
         <v>130</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="H8" s="13" t="s">
         <v>73</v>
@@ -2487,7 +2527,7 @@
         <v>12</v>
       </c>
       <c r="K8" s="13" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="L8" s="7" t="n">
         <f aca="false">IF(A8="","",IF(K8="50/50",0.5,IF(K8="Prorata salaires",Paramètres!$B$9,IF(K8="Personne 1 seul",1,IF(K8="Personne 2 seul",0,0.5)))))</f>
@@ -2504,13 +2544,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D9" s="13" t="s">
         <v>36</v>
@@ -2523,7 +2563,7 @@
         <v>40</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="H9" s="13" t="s">
         <v>79</v>
@@ -2533,7 +2573,7 @@
         <v>14</v>
       </c>
       <c r="K9" s="13" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="L9" s="7" t="n">
         <f aca="false">IF(A9="","",IF(K9="50/50",0.5,IF(K9="Prorata salaires",Paramètres!$B$9,IF(K9="Personne 1 seul",1,IF(K9="Personne 2 seul",0,0.5)))))</f>
@@ -2550,10 +2590,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="C10" s="13" t="s">
         <v>28</v>
@@ -2569,7 +2609,7 @@
         <v>30</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="H10" s="13" t="s">
         <v>79</v>
@@ -2579,7 +2619,7 @@
         <v>10</v>
       </c>
       <c r="K10" s="13" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="L10" s="7" t="n">
         <f aca="false">IF(A10="","",IF(K10="50/50",0.5,IF(K10="Prorata salaires",Paramètres!$B$9,IF(K10="Personne 1 seul",1,IF(K10="Personne 2 seul",0,0.5)))))</f>
@@ -2596,10 +2636,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C11" s="13" t="s">
         <v>28</v>
@@ -2615,7 +2655,7 @@
         <v>70</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="H11" s="13" t="s">
         <v>77</v>
@@ -2625,7 +2665,7 @@
         <v>1</v>
       </c>
       <c r="K11" s="13" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="L11" s="7" t="n">
         <f aca="false">IF(A11="","",IF(K11="50/50",0.5,IF(K11="Prorata salaires",Paramètres!$B$9,IF(K11="Personne 1 seul",1,IF(K11="Personne 2 seul",0,0.5)))))</f>
@@ -2642,10 +2682,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>28</v>
@@ -2661,7 +2701,7 @@
         <v>28</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="H12" s="13" t="s">
         <v>44</v>
@@ -2671,7 +2711,7 @@
         <v>8</v>
       </c>
       <c r="K12" s="13" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="L12" s="7" t="n">
         <f aca="false">IF(A12="","",IF(K12="50/50",0.5,IF(K12="Prorata salaires",Paramètres!$B$9,IF(K12="Personne 1 seul",1,IF(K12="Personne 2 seul",0,0.5)))))</f>
@@ -2688,13 +2728,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D13" s="13" t="s">
         <v>36</v>
@@ -2707,7 +2747,7 @@
         <v>600</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="H13" s="13" t="s">
         <v>77</v>
@@ -2715,7 +2755,7 @@
       <c r="I13" s="13"/>
       <c r="J13" s="13"/>
       <c r="K13" s="13" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="L13" s="7" t="n">
         <f aca="false">IF(A13="","",IF(K13="50/50",0.5,IF(K13="Prorata salaires",Paramètres!$B$9,IF(K13="Personne 1 seul",1,IF(K13="Personne 2 seul",0,0.5)))))</f>
@@ -2732,7 +2772,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="B14" s="13" t="s">
         <v>82</v>
@@ -2751,7 +2791,7 @@
         <v>150</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="H14" s="13" t="s">
         <v>77</v>
@@ -2763,7 +2803,7 @@
         <v>3</v>
       </c>
       <c r="K14" s="13" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="L14" s="7" t="n">
         <f aca="false">IF(A14="","",IF(K14="50/50",0.5,IF(K14="Prorata salaires",Paramètres!$B$9,IF(K14="Personne 1 seul",1,IF(K14="Personne 2 seul",0,0.5)))))</f>
@@ -2780,13 +2820,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D15" s="13" t="s">
         <v>36</v>
@@ -2799,19 +2839,19 @@
         <v>90</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="H15" s="13" t="s">
         <v>77</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="J15" s="13" t="n">
         <v>28</v>
       </c>
       <c r="K15" s="13" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="L15" s="7" t="n">
         <f aca="false">IF(A15="","",IF(K15="50/50",0.5,IF(K15="Prorata salaires",Paramètres!$B$9,IF(K15="Personne 1 seul",1,IF(K15="Personne 2 seul",0,0.5)))))</f>
@@ -2828,13 +2868,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D16" s="13" t="s">
         <v>45</v>
@@ -2847,7 +2887,7 @@
         <v>50</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="H16" s="13" t="s">
         <v>77</v>
@@ -2855,7 +2895,7 @@
       <c r="I16" s="13"/>
       <c r="J16" s="13"/>
       <c r="K16" s="13" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="L16" s="7" t="n">
         <f aca="false">IF(A16="","",IF(K16="50/50",0.5,IF(K16="Prorata salaires",Paramètres!$B$9,IF(K16="Personne 1 seul",1,IF(K16="Personne 2 seul",0,0.5)))))</f>
@@ -2872,13 +2912,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D17" s="13" t="s">
         <v>36</v>
@@ -2891,7 +2931,7 @@
         <v>30</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="H17" s="13" t="s">
         <v>77</v>
@@ -2899,7 +2939,7 @@
       <c r="I17" s="13"/>
       <c r="J17" s="13"/>
       <c r="K17" s="13" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="L17" s="7" t="n">
         <f aca="false">IF(A17="","",IF(K17="50/50",0.5,IF(K17="Prorata salaires",Paramètres!$B$9,IF(K17="Personne 1 seul",1,IF(K17="Personne 2 seul",0,0.5)))))</f>
@@ -2916,13 +2956,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D18" s="13" t="s">
         <v>45</v>
@@ -2935,7 +2975,7 @@
         <v>41.6666666666667</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="H18" s="13" t="s">
         <v>77</v>
@@ -2943,7 +2983,7 @@
       <c r="I18" s="13"/>
       <c r="J18" s="13"/>
       <c r="K18" s="13" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="L18" s="7" t="n">
         <f aca="false">IF(A18="","",IF(K18="50/50",0.5,IF(K18="Prorata salaires",Paramètres!$B$9,IF(K18="Personne 1 seul",1,IF(K18="Personne 2 seul",0,0.5)))))</f>
@@ -2960,13 +3000,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D19" s="13" t="s">
         <v>36</v>
@@ -2980,7 +3020,7 @@
         <v>129</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="H19" s="13" t="s">
         <v>77</v>
@@ -2992,7 +3032,7 @@
         <v>3</v>
       </c>
       <c r="K19" s="13" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="L19" s="7" t="n">
         <f aca="false">IF(A19="","",IF(K19="50/50",0.5,IF(K19="Prorata salaires",Paramètres!$B$9,IF(K19="Personne 1 seul",1,IF(K19="Personne 2 seul",0,0.5)))))</f>
@@ -3009,10 +3049,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>134</v>
+        <v>82</v>
       </c>
       <c r="C20" s="13" t="s">
         <v>28</v>
@@ -3021,24 +3061,26 @@
         <v>36</v>
       </c>
       <c r="E20" s="18" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="F20" s="6" t="n">
         <f aca="false">IF(A20="","",IFERROR(E20/INDEX(Paramètres!$E$4:$E$7,MATCH(D20,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="H20" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="I20" s="13"/>
+      <c r="I20" s="13" t="s">
+        <v>86</v>
+      </c>
       <c r="J20" s="13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K20" s="13" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="L20" s="7" t="n">
         <f aca="false">IF(A20="","",IF(K20="50/50",0.5,IF(K20="Prorata salaires",Paramètres!$B$9,IF(K20="Personne 1 seul",1,IF(K20="Personne 2 seul",0,0.5)))))</f>
@@ -3046,19 +3088,19 @@
       </c>
       <c r="M20" s="6" t="n">
         <f aca="false">IF(A20="","",F20*L20)</f>
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="N20" s="6" t="n">
         <f aca="false">IF(A20="","",F20-M20)</f>
-        <v>60</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>123</v>
+        <v>82</v>
       </c>
       <c r="C21" s="13" t="s">
         <v>28</v>
@@ -3067,24 +3109,26 @@
         <v>36</v>
       </c>
       <c r="E21" s="18" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F21" s="6" t="n">
         <f aca="false">IF(A21="","",IFERROR(E21/INDEX(Paramètres!$E$4:$E$7,MATCH(D21,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="H21" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="I21" s="13"/>
+      <c r="I21" s="13" t="s">
+        <v>89</v>
+      </c>
       <c r="J21" s="13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K21" s="13" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="L21" s="7" t="n">
         <f aca="false">IF(A21="","",IF(K21="50/50",0.5,IF(K21="Prorata salaires",Paramètres!$B$9,IF(K21="Personne 1 seul",1,IF(K21="Personne 2 seul",0,0.5)))))</f>
@@ -3092,43 +3136,45 @@
       </c>
       <c r="M21" s="6" t="n">
         <f aca="false">IF(A21="","",F21*L21)</f>
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="N21" s="6" t="n">
         <f aca="false">IF(A21="","",F21-M21)</f>
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>108</v>
+        <v>28</v>
       </c>
       <c r="D22" s="13" t="s">
         <v>36</v>
       </c>
       <c r="E22" s="18" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="F22" s="6" t="n">
         <f aca="false">IF(A22="","",IFERROR(E22/INDEX(Paramètres!$E$4:$E$7,MATCH(D22,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="H22" s="13" t="s">
         <v>77</v>
       </c>
       <c r="I22" s="13"/>
-      <c r="J22" s="13"/>
+      <c r="J22" s="13" t="n">
+        <v>1</v>
+      </c>
       <c r="K22" s="13" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="L22" s="7" t="n">
         <f aca="false">IF(A22="","",IF(K22="50/50",0.5,IF(K22="Prorata salaires",Paramètres!$B$9,IF(K22="Personne 1 seul",1,IF(K22="Personne 2 seul",0,0.5)))))</f>
@@ -3136,67 +3182,101 @@
       </c>
       <c r="M22" s="6" t="n">
         <f aca="false">IF(A22="","",F22*L22)</f>
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="N22" s="6" t="n">
         <f aca="false">IF(A22="","",F22-M22)</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E23" s="18" t="n">
         <v>30</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="13"/>
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="6" t="str">
+      <c r="F23" s="6" t="n">
         <f aca="false">IF(A23="","",IFERROR(E23/INDEX(Paramètres!$E$4:$E$7,MATCH(D23,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v/>
-      </c>
-      <c r="G23" s="13"/>
-      <c r="H23" s="13"/>
+        <v>30</v>
+      </c>
+      <c r="G23" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="H23" s="13" t="s">
+        <v>77</v>
+      </c>
       <c r="I23" s="13"/>
-      <c r="J23" s="13"/>
-      <c r="K23" s="13"/>
-      <c r="L23" s="7" t="str">
+      <c r="J23" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="L23" s="7" t="n">
         <f aca="false">IF(A23="","",IF(K23="50/50",0.5,IF(K23="Prorata salaires",Paramètres!$B$9,IF(K23="Personne 1 seul",1,IF(K23="Personne 2 seul",0,0.5)))))</f>
-        <v/>
-      </c>
-      <c r="M23" s="6" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="M23" s="6" t="n">
         <f aca="false">IF(A23="","",F23*L23)</f>
-        <v/>
-      </c>
-      <c r="N23" s="6" t="str">
+        <v>15</v>
+      </c>
+      <c r="N23" s="6" t="n">
         <f aca="false">IF(A23="","",F23-M23)</f>
-        <v/>
+        <v>15</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="13"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="6" t="str">
+      <c r="A24" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E24" s="18" t="n">
+        <v>60</v>
+      </c>
+      <c r="F24" s="6" t="n">
         <f aca="false">IF(A24="","",IFERROR(E24/INDEX(Paramètres!$E$4:$E$7,MATCH(D24,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v/>
-      </c>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
+        <v>60</v>
+      </c>
+      <c r="G24" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="H24" s="13" t="s">
+        <v>77</v>
+      </c>
       <c r="I24" s="13"/>
       <c r="J24" s="13"/>
-      <c r="K24" s="13"/>
-      <c r="L24" s="7" t="str">
+      <c r="K24" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="L24" s="7" t="n">
         <f aca="false">IF(A24="","",IF(K24="50/50",0.5,IF(K24="Prorata salaires",Paramètres!$B$9,IF(K24="Personne 1 seul",1,IF(K24="Personne 2 seul",0,0.5)))))</f>
-        <v/>
-      </c>
-      <c r="M24" s="6" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="M24" s="6" t="n">
         <f aca="false">IF(A24="","",F24*L24)</f>
-        <v/>
-      </c>
-      <c r="N24" s="6" t="str">
+        <v>30</v>
+      </c>
+      <c r="N24" s="6" t="n">
         <f aca="false">IF(A24="","",F24-M24)</f>
-        <v/>
+        <v>30</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4041,37 +4121,37 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="22" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="F55" s="9" t="n">
         <f aca="false">SUM(F5:F54)</f>
-        <v>2902</v>
+        <v>3002</v>
       </c>
       <c r="M55" s="9" t="n">
         <f aca="false">SUM(M5:M54)</f>
-        <v>1545.15891472868</v>
+        <v>1595.15891472868</v>
       </c>
       <c r="N55" s="9" t="n">
         <f aca="false">SUM(N5:N54)</f>
-        <v>1356.84108527132</v>
+        <v>1406.84108527132</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H54" type="list">
-      <formula1>Comptes!$A$5:$A$14</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C5:C54" type="list">
+      <formula1>"Fixe,Variable"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D54" type="list">
       <formula1>"Mensuelle,Trimestrielle,Semestrielle,Annuelle"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C5:C54" type="list">
-      <formula1>"Fixe,Variable"</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G54" type="list">
+      <formula1>"Prélèvement,Virement,Carte,Chèque,Espèces"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G54" type="list">
-      <formula1>"Prélèvement,Virement,Carte,Chèque,Espèces"</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H54" type="list">
+      <formula1>Comptes!$A$5:$A$14</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K5:K54" type="list">
@@ -4108,17 +4188,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>18</v>
@@ -4127,27 +4207,27 @@
         <v>3</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>32</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>35</v>
@@ -4171,10 +4251,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>38</v>
@@ -4198,13 +4278,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="D7" s="18" t="n">
         <v>140</v>
@@ -4225,13 +4305,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="D8" s="18" t="n">
         <v>270</v>
@@ -4460,7 +4540,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="22" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="F25" s="9" t="n">
         <f aca="false">SUM(F5:F24)</f>
@@ -4511,52 +4591,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="B5" s="13" t="s">
         <v>35</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>36</v>
@@ -4569,7 +4649,7 @@
         <v>35</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="H5" s="13" t="s">
         <v>41</v>
@@ -4580,13 +4660,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>35</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="D6" s="13" t="s">
         <v>39</v>
@@ -4599,7 +4679,7 @@
         <v>40</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="H6" s="13" t="s">
         <v>41</v>
@@ -4608,13 +4688,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="B7" s="13" t="s">
         <v>35</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="D7" s="13" t="s">
         <v>36</v>
@@ -4627,7 +4707,7 @@
         <v>11</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="H7" s="13" t="s">
         <v>41</v>
@@ -5156,7 +5236,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="22" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="F45" s="9" t="n">
         <f aca="false">SUM(F5:F44)</f>
@@ -5208,17 +5288,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="23" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="B4" s="6" t="n">
         <f aca="false">SUMIFS(Charges!$F$5:$F$54,Charges!$B$5:$B$54,"Imprévus")</f>
@@ -5227,7 +5307,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="B5" s="24" t="n">
         <v>46266</v>
@@ -5235,7 +5315,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>0</v>
@@ -5243,7 +5323,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="B7" s="25" t="n">
         <f aca="true">IF(B5="",0,MAX(0,(YEAR(TODAY())-YEAR(B5))*12+MONTH(TODAY())-MONTH(B5)+1))</f>
@@ -5252,7 +5332,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="B8" s="6" t="n">
         <f aca="false">B6+B4*B7</f>
@@ -5261,7 +5341,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">SUM(C13:C62)</f>
@@ -5270,7 +5350,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">B8-B9</f>
@@ -5279,21 +5359,21 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5301,7 +5381,7 @@
         <v>46285</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="C13" s="18" t="n">
         <v>220</v>
@@ -5315,7 +5395,7 @@
         <v>46300</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="C14" s="18" t="n">
         <v>85</v>

</xml_diff>

<commit_message>
Correction des textes d'aide (v1.0.1) et ligne Provision imprévus dans le vierge
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KqkJNWVZSWN9upSPoUaH5h
</commit_message>
<xml_diff>
--- a/suivi_comptes_example.xlsx
+++ b/suivi_comptes_example.xlsx
@@ -31,7 +31,7 @@
     <t xml:space="preserve">Synthèse mensuelle</t>
   </si>
   <si>
-    <t xml:space="preserve">Tout est calculé à partir des onglets Charges, Revenus et Comptes. Ne rien saisir ici.</t>
+    <t xml:space="preserve">Tout est calculé à partir des autres onglets (Paramètres, Comptes, Charges, Revenus, Charges perso). Ne rien saisir ici.</t>
   </si>
   <si>
     <t xml:space="preserve">1. Par personne</t>
@@ -106,7 +106,7 @@
     <t xml:space="preserve">Total</t>
   </si>
   <si>
-    <t xml:space="preserve">Lecture : un compte joint à solde 0 est équilibré. Un compte perso à solde positif = reste à vivre ; négatif = salaire insuffisant. Les aides sont réparties sur les deux personnes au prorata de leurs parts de charges (hypothèse).</t>
+    <t xml:space="preserve">Lecture : un compte joint à solde 0 est équilibré. Un compte perso à solde positif = reste après charges communes (avant charges perso et épargne perso, voir tableau 1) ; négatif = salaire insuffisant. Un compte d'épargne affiche les virements reçus ce mois. Les aides sont réparties sur les deux personnes au prorata de leurs parts de charges (hypothèse).</t>
   </si>
   <si>
     <t xml:space="preserve">3. Charges communes : fixe vs variable (mensuel)</t>
@@ -169,7 +169,7 @@
     <t xml:space="preserve">Part de la Personne 1 dans les salaires (pour « Prorata salaires »)</t>
   </si>
   <si>
-    <t xml:space="preserve">Hypothèse : 50 % si aucun salaire n'est saisi.</t>
+    <t xml:space="preserve">Hypothèse : 50 % si aucun salaire n'est saisi. Le prénom des salaires (onglet Revenus) doit être identique à celui saisi plus haut.</t>
   </si>
   <si>
     <t xml:space="preserve">Modes de répartition possibles : 50/50 · Prorata salaires · Personne 1 seul · Personne 2 seul</t>
@@ -199,7 +199,7 @@
     <t xml:space="preserve">Montant</t>
   </si>
   <si>
-    <t xml:space="preserve">Épargne perso : pourcentage du reste (si Pourcentage)</t>
+    <t xml:space="preserve">Épargne perso : pourcentage du reste après charges perso (si Pourcentage)</t>
   </si>
   <si>
     <t xml:space="preserve">Épargne perso : montant €/mois (si Montant)</t>
@@ -211,13 +211,13 @@
     <t xml:space="preserve">Provision imprévus (% des salaires du foyer)</t>
   </si>
   <si>
-    <t xml:space="preserve">Alimente la ligne « Provision imprévus » de l'onglet Charges (réparties 50/50, sur le compte joint indiqué).</t>
+    <t xml:space="preserve">Le montant de la ligne « Provision imprévus » de l'onglet Charges vaut ce pourcentage × les salaires mensuels du foyer. Les comptes (débité et destinataire) et la répartition de cette ligne sont à régler dans Charges.</t>
   </si>
   <si>
     <t xml:space="preserve">Version du modèle</t>
   </si>
   <si>
-    <t xml:space="preserve">1.0.0</t>
+    <t xml:space="preserve">1.0.1</t>
   </si>
   <si>
     <t xml:space="preserve">Voir MIGRATION.md pour migrer un fichier d'une version à l'autre.</t>
@@ -226,7 +226,7 @@
     <t xml:space="preserve">Comptes bancaires</t>
   </si>
   <si>
-    <t xml:space="preserve">Paramétrez ici vos comptes (10 lignes). Le nom saisi ici alimente les listes déroulantes des autres onglets.</t>
+    <t xml:space="preserve">Paramétrez ici vos comptes (10 lignes). Le nom saisi ici alimente les listes déroulantes des autres onglets. Si vous renommez un compte, corrigez-le aussi dans les lignes déjà saisies.</t>
   </si>
   <si>
     <t xml:space="preserve">Nom du compte</t>
@@ -472,7 +472,7 @@
     <t xml:space="preserve">Revenus et aides</t>
   </si>
   <si>
-    <t xml:space="preserve">Salaires (arrivent sur le compte de chacun) et aides type CAF (peuvent arriver sur un compte joint). 20 lignes.</t>
+    <t xml:space="preserve">Salaires (arrivent sur le compte de chacun) et aides type CAF (peuvent arriver sur un compte joint). 20 lignes. Colonne Personne : prénom identique à Paramètres (obligatoire pour un salaire), ou « Commun ».</t>
   </si>
   <si>
     <t xml:space="preserve">Compte de réception</t>
@@ -523,7 +523,7 @@
     <t xml:space="preserve">Notez chaque dépense imprévue ici (date, libellé, montant). Le solde de la provision se met à jour tout seul.</t>
   </si>
   <si>
-    <t xml:space="preserve">Provision mensuelle (ligne « Imprévus » de Charges)</t>
+    <t xml:space="preserve">Provision mensuelle (somme des lignes de catégorie « Imprévus » dans Charges)</t>
   </si>
   <si>
     <t xml:space="preserve">Début du suivi (1er du mois)</t>

</xml_diff>

<commit_message>
Solde des comptes perso : prise en compte des charges perso et de l'épargne perso (v1.1.0)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KqkJNWVZSWN9upSPoUaH5h
</commit_message>
<xml_diff>
--- a/suivi_comptes_example.xlsx
+++ b/suivi_comptes_example.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="181">
   <si>
     <t xml:space="preserve">Synthèse mensuelle</t>
   </si>
@@ -100,13 +100,19 @@
     <t xml:space="preserve">Participations versées (vers comptes joints)</t>
   </si>
   <si>
+    <t xml:space="preserve">Solde avant charges perso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charges perso &amp; épargne perso débitées</t>
+  </si>
+  <si>
     <t xml:space="preserve">Solde mensuel prévisionnel</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
   </si>
   <si>
-    <t xml:space="preserve">Lecture : un compte joint à solde 0 est équilibré. Un compte perso à solde positif = reste après charges communes (avant charges perso et épargne perso, voir tableau 1) ; négatif = salaire insuffisant. Un compte d'épargne affiche les virements reçus ce mois. Les aides sont réparties sur les deux personnes au prorata de leurs parts de charges (hypothèse).</t>
+    <t xml:space="preserve">Lecture : un compte joint à solde 0 est équilibré. Un compte perso à solde positif = ce qu'il reste après charges communes, charges perso (détail ou forfait) et épargne perso, imputées à ce compte (compte débité de la ligne, sinon le compte perso) ; négatif = salaire insuffisant. Un compte d'épargne affiche les virements reçus ce mois. Les aides sont réparties sur les deux personnes au prorata de leurs parts de charges (hypothèse).</t>
   </si>
   <si>
     <t xml:space="preserve">3. Charges communes : fixe vs variable (mensuel)</t>
@@ -217,7 +223,7 @@
     <t xml:space="preserve">Version du modèle</t>
   </si>
   <si>
-    <t xml:space="preserve">1.0.1</t>
+    <t xml:space="preserve">1.1.0</t>
   </si>
   <si>
     <t xml:space="preserve">Voir MIGRATION.md pour migrer un fichier d'une version à l'autre.</t>
@@ -502,7 +508,10 @@
     <t xml:space="preserve">Charges personnelles (facultatif)</t>
   </si>
   <si>
-    <t xml:space="preserve">Dépenses propres à chacun. Utilisé seulement si le mode « Détail » est choisi pour la personne dans Paramètres.</t>
+    <t xml:space="preserve">Dépenses propres à chacun. Utilisé seulement si le mode « Détail » est choisi pour la personne dans Paramètres. Compte débité : si vide, la dépense est imputée au compte perso de la personne.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compte imputé (calculé)</t>
   </si>
   <si>
     <t xml:space="preserve">Salle de sport</t>
@@ -1104,7 +1113,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -1114,7 +1123,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1347,6 +1358,12 @@
       <c r="J12" s="4" t="s">
         <v>24</v>
       </c>
+      <c r="K12" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="str">
@@ -1389,6 +1406,14 @@
         <f aca="false">IF($A13="","",G13+D13+H13+IF(B13="Joint",E13+F13,0)-C13-I13)</f>
         <v>925.314793340221</v>
       </c>
+      <c r="K13" s="6" t="n">
+        <f aca="false">IF($A13="","",SUMIFS('Charges perso'!$F$5:$F$44,'Charges perso'!$J$5:$J$44,$A13)+IF(AND($A13=Paramètres!$B$6,Paramètres!$B$15="Forfait"),Paramètres!$B$16,0)+IF(AND($A13=Paramètres!$B$7,Paramètres!$C$15="Forfait"),Paramètres!$C$16,0)+IF($A13=Paramètres!$B$6,$J$5,0)+IF($A13=Paramètres!$B$7,$J$6,0))</f>
+        <v>337.794438002066</v>
+      </c>
+      <c r="L13" s="6" t="n">
+        <f aca="false">IF($A13="","",J13-K13)</f>
+        <v>587.520355338154</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="str">
@@ -1431,6 +1456,14 @@
         <f aca="false">IF($A14="","",G14+D14+H14+IF(B14="Joint",E14+F14,0)-C14-I14)</f>
         <v>602.685206659779</v>
       </c>
+      <c r="K14" s="6" t="n">
+        <f aca="false">IF($A14="","",SUMIFS('Charges perso'!$F$5:$F$44,'Charges perso'!$J$5:$J$44,$A14)+IF(AND($A14=Paramètres!$B$6,Paramètres!$B$15="Forfait"),Paramètres!$B$16,0)+IF(AND($A14=Paramètres!$B$7,Paramètres!$C$15="Forfait"),Paramètres!$C$16,0)+IF($A14=Paramètres!$B$6,$J$5,0)+IF($A14=Paramètres!$B$7,$J$6,0))</f>
+        <v>550</v>
+      </c>
+      <c r="L14" s="6" t="n">
+        <f aca="false">IF($A14="","",J14-K14)</f>
+        <v>52.6852066597792</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="str">
@@ -1473,6 +1506,14 @@
         <f aca="false">IF($A15="","",G15+D15+H15+IF(B15="Joint",E15+F15,0)-C15-I15)</f>
         <v>0</v>
       </c>
+      <c r="K15" s="6" t="n">
+        <f aca="false">IF($A15="","",SUMIFS('Charges perso'!$F$5:$F$44,'Charges perso'!$J$5:$J$44,$A15)+IF(AND($A15=Paramètres!$B$6,Paramètres!$B$15="Forfait"),Paramètres!$B$16,0)+IF(AND($A15=Paramètres!$B$7,Paramètres!$C$15="Forfait"),Paramètres!$C$16,0)+IF($A15=Paramètres!$B$6,$J$5,0)+IF($A15=Paramètres!$B$7,$J$6,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <f aca="false">IF($A15="","",J15-K15)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="str">
@@ -1515,6 +1556,14 @@
         <f aca="false">IF($A16="","",G16+D16+H16+IF(B16="Joint",E16+F16,0)-C16-I16)</f>
         <v>0</v>
       </c>
+      <c r="K16" s="6" t="n">
+        <f aca="false">IF($A16="","",SUMIFS('Charges perso'!$F$5:$F$44,'Charges perso'!$J$5:$J$44,$A16)+IF(AND($A16=Paramètres!$B$6,Paramètres!$B$15="Forfait"),Paramètres!$B$16,0)+IF(AND($A16=Paramètres!$B$7,Paramètres!$C$15="Forfait"),Paramètres!$C$16,0)+IF($A16=Paramètres!$B$6,$J$5,0)+IF($A16=Paramètres!$B$7,$J$6,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L16" s="6" t="n">
+        <f aca="false">IF($A16="","",J16-K16)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="str">
@@ -1557,6 +1606,14 @@
         <f aca="false">IF($A17="","",G17+D17+H17+IF(B17="Joint",E17+F17,0)-C17-I17)</f>
         <v>0</v>
       </c>
+      <c r="K17" s="6" t="n">
+        <f aca="false">IF($A17="","",SUMIFS('Charges perso'!$F$5:$F$44,'Charges perso'!$J$5:$J$44,$A17)+IF(AND($A17=Paramètres!$B$6,Paramètres!$B$15="Forfait"),Paramètres!$B$16,0)+IF(AND($A17=Paramètres!$B$7,Paramètres!$C$15="Forfait"),Paramètres!$C$16,0)+IF($A17=Paramètres!$B$6,$J$5,0)+IF($A17=Paramètres!$B$7,$J$6,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L17" s="6" t="n">
+        <f aca="false">IF($A17="","",J17-K17)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="str">
@@ -1599,6 +1656,14 @@
         <f aca="false">IF($A18="","",G18+D18+H18+IF(B18="Joint",E18+F18,0)-C18-I18)</f>
         <v>150</v>
       </c>
+      <c r="K18" s="6" t="n">
+        <f aca="false">IF($A18="","",SUMIFS('Charges perso'!$F$5:$F$44,'Charges perso'!$J$5:$J$44,$A18)+IF(AND($A18=Paramètres!$B$6,Paramètres!$B$15="Forfait"),Paramètres!$B$16,0)+IF(AND($A18=Paramètres!$B$7,Paramètres!$C$15="Forfait"),Paramètres!$C$16,0)+IF($A18=Paramètres!$B$6,$J$5,0)+IF($A18=Paramètres!$B$7,$J$6,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L18" s="6" t="n">
+        <f aca="false">IF($A18="","",J18-K18)</f>
+        <v>150</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="str">
@@ -1641,6 +1706,14 @@
         <f aca="false">IF($A19="","",G19+D19+H19+IF(B19="Joint",E19+F19,0)-C19-I19)</f>
         <v>129</v>
       </c>
+      <c r="K19" s="6" t="n">
+        <f aca="false">IF($A19="","",SUMIFS('Charges perso'!$F$5:$F$44,'Charges perso'!$J$5:$J$44,$A19)+IF(AND($A19=Paramètres!$B$6,Paramètres!$B$15="Forfait"),Paramètres!$B$16,0)+IF(AND($A19=Paramètres!$B$7,Paramètres!$C$15="Forfait"),Paramètres!$C$16,0)+IF($A19=Paramètres!$B$6,$J$5,0)+IF($A19=Paramètres!$B$7,$J$6,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L19" s="6" t="n">
+        <f aca="false">IF($A19="","",J19-K19)</f>
+        <v>129</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="str">
@@ -1683,6 +1756,14 @@
         <f aca="false">IF($A20="","",G20+D20+H20+IF(B20="Joint",E20+F20,0)-C20-I20)</f>
         <v>50</v>
       </c>
+      <c r="K20" s="6" t="n">
+        <f aca="false">IF($A20="","",SUMIFS('Charges perso'!$F$5:$F$44,'Charges perso'!$J$5:$J$44,$A20)+IF(AND($A20=Paramètres!$B$6,Paramètres!$B$15="Forfait"),Paramètres!$B$16,0)+IF(AND($A20=Paramètres!$B$7,Paramètres!$C$15="Forfait"),Paramètres!$C$16,0)+IF($A20=Paramètres!$B$6,$J$5,0)+IF($A20=Paramètres!$B$7,$J$6,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L20" s="6" t="n">
+        <f aca="false">IF($A20="","",J20-K20)</f>
+        <v>50</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="str">
@@ -1725,6 +1806,14 @@
         <f aca="false">IF($A21="","",G21+D21+H21+IF(B21="Joint",E21+F21,0)-C21-I21)</f>
         <v>50</v>
       </c>
+      <c r="K21" s="6" t="n">
+        <f aca="false">IF($A21="","",SUMIFS('Charges perso'!$F$5:$F$44,'Charges perso'!$J$5:$J$44,$A21)+IF(AND($A21=Paramètres!$B$6,Paramètres!$B$15="Forfait"),Paramètres!$B$16,0)+IF(AND($A21=Paramètres!$B$7,Paramètres!$C$15="Forfait"),Paramètres!$C$16,0)+IF($A21=Paramètres!$B$6,$J$5,0)+IF($A21=Paramètres!$B$7,$J$6,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L21" s="6" t="n">
+        <f aca="false">IF($A21="","",J21-K21)</f>
+        <v>50</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="str">
@@ -1767,10 +1856,18 @@
         <f aca="false">IF($A22="","",G22+D22+H22+IF(B22="Joint",E22+F22,0)-C22-I22)</f>
         <v/>
       </c>
+      <c r="K22" s="6" t="str">
+        <f aca="false">IF($A22="","",SUMIFS('Charges perso'!$F$5:$F$44,'Charges perso'!$J$5:$J$44,$A22)+IF(AND($A22=Paramètres!$B$6,Paramètres!$B$15="Forfait"),Paramètres!$B$16,0)+IF(AND($A22=Paramètres!$B$7,Paramètres!$C$15="Forfait"),Paramètres!$C$16,0)+IF($A22=Paramètres!$B$6,$J$5,0)+IF($A22=Paramètres!$B$7,$J$6,0))</f>
+        <v/>
+      </c>
+      <c r="L22" s="6" t="str">
+        <f aca="false">IF($A22="","",J22-K22)</f>
+        <v/>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="9" t="n">
@@ -1805,20 +1902,28 @@
         <f aca="false">SUM(J13:J22)</f>
         <v>1907</v>
       </c>
+      <c r="K23" s="9" t="n">
+        <f aca="false">SUM(K13:K22)</f>
+        <v>887.794438002066</v>
+      </c>
+      <c r="L23" s="9" t="n">
+        <f aca="false">SUM(L13:L22)</f>
+        <v>1019.20556199793</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B28" s="6" t="n">
         <f aca="false">SUMIFS(Charges!$F$5:$F$54,Charges!$C$5:$C$54,"Fixe")</f>
@@ -1831,7 +1936,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B29" s="6" t="n">
         <f aca="false">SUMIFS(Charges!$F$5:$F$54,Charges!$C$5:$C$54,"Variable")</f>
@@ -1844,7 +1949,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B30" s="9" t="n">
         <f aca="false">B28+B29</f>
@@ -1882,31 +1987,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D3" s="12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E4" s="5" t="n">
         <v>1</v>
@@ -1914,13 +2019,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>3</v>
@@ -1928,13 +2033,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>6</v>
@@ -1942,13 +2047,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>12</v>
@@ -1956,7 +2061,7 @@
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B9" s="15" t="n">
         <f aca="false">IFERROR(SUMIFS(Revenus!$F$5:$F$24,Revenus!$B$5:$B$24,"Salaire",Revenus!$C$5:$C$24,$B$4)/SUMIFS(Revenus!$F$5:$F$24,Revenus!$B$5:$B$24,"Salaire"),0.5)</f>
@@ -1965,17 +2070,17 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B14" s="16" t="str">
         <f aca="false">$B$4</f>
@@ -1988,18 +2093,18 @@
     </row>
     <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="17" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B16" s="18" t="n">
         <v>0</v>
@@ -2010,18 +2115,18 @@
     </row>
     <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="17" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B18" s="19" t="n">
         <v>0.3</v>
@@ -2032,7 +2137,7 @@
     </row>
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B19" s="18" t="n">
         <v>0</v>
@@ -2043,12 +2148,12 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B22" s="20" t="n">
         <v>0.03</v>
@@ -2056,20 +2161,20 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -2109,152 +2214,152 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>18</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C8" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="B8" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>75</v>
-      </c>
       <c r="D8" s="13" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="B11" s="13" t="s">
-        <v>82</v>
-      </c>
       <c r="C11" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2304,50 +2409,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="M4" s="4" t="str">
         <f aca="false">"Part "&amp;Paramètres!$B$4&amp;" (€/mois)"</f>
@@ -2360,16 +2465,16 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E5" s="18" t="n">
         <v>1150</v>
@@ -2379,17 +2484,17 @@
         <v>1150</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I5" s="13"/>
       <c r="J5" s="13" t="n">
         <v>5</v>
       </c>
       <c r="K5" s="13" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="L5" s="7" t="n">
         <f aca="false">IF(A5="","",IF(K5="50/50",0.5,IF(K5="Prorata salaires",Paramètres!$B$9,IF(K5="Personne 1 seul",1,IF(K5="Personne 2 seul",0,0.5)))))</f>
@@ -2406,16 +2511,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E6" s="18" t="n">
         <v>45</v>
@@ -2425,17 +2530,17 @@
         <v>45</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H6" s="13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I6" s="13"/>
       <c r="J6" s="13" t="n">
         <v>5</v>
       </c>
       <c r="K6" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L6" s="7" t="n">
         <f aca="false">IF(A6="","",IF(K6="50/50",0.5,IF(K6="Prorata salaires",Paramètres!$B$9,IF(K6="Personne 1 seul",1,IF(K6="Personne 2 seul",0,0.5)))))</f>
@@ -2452,16 +2557,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E7" s="18" t="n">
         <v>1300</v>
@@ -2471,17 +2576,17 @@
         <v>108.333333333333</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H7" s="13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I7" s="13"/>
       <c r="J7" s="13" t="n">
         <v>15</v>
       </c>
       <c r="K7" s="13" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="L7" s="7" t="n">
         <f aca="false">IF(A7="","",IF(K7="50/50",0.5,IF(K7="Prorata salaires",Paramètres!$B$9,IF(K7="Personne 1 seul",1,IF(K7="Personne 2 seul",0,0.5)))))</f>
@@ -2498,16 +2603,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E8" s="18" t="n">
         <v>130</v>
@@ -2517,17 +2622,17 @@
         <v>130</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H8" s="13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I8" s="13"/>
       <c r="J8" s="13" t="n">
         <v>12</v>
       </c>
       <c r="K8" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L8" s="7" t="n">
         <f aca="false">IF(A8="","",IF(K8="50/50",0.5,IF(K8="Prorata salaires",Paramètres!$B$9,IF(K8="Personne 1 seul",1,IF(K8="Personne 2 seul",0,0.5)))))</f>
@@ -2544,16 +2649,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="B9" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="B9" s="13" t="s">
-        <v>113</v>
-      </c>
       <c r="C9" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E9" s="18" t="n">
         <v>40</v>
@@ -2563,17 +2668,17 @@
         <v>40</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I9" s="13"/>
       <c r="J9" s="13" t="n">
         <v>14</v>
       </c>
       <c r="K9" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L9" s="7" t="n">
         <f aca="false">IF(A9="","",IF(K9="50/50",0.5,IF(K9="Prorata salaires",Paramètres!$B$9,IF(K9="Personne 1 seul",1,IF(K9="Personne 2 seul",0,0.5)))))</f>
@@ -2590,16 +2695,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E10" s="18" t="n">
         <v>30</v>
@@ -2609,17 +2714,17 @@
         <v>30</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I10" s="13"/>
       <c r="J10" s="13" t="n">
         <v>10</v>
       </c>
       <c r="K10" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L10" s="7" t="n">
         <f aca="false">IF(A10="","",IF(K10="50/50",0.5,IF(K10="Prorata salaires",Paramètres!$B$9,IF(K10="Personne 1 seul",1,IF(K10="Personne 2 seul",0,0.5)))))</f>
@@ -2636,16 +2741,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E11" s="18" t="n">
         <v>210</v>
@@ -2655,17 +2760,17 @@
         <v>70</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I11" s="13"/>
       <c r="J11" s="13" t="n">
         <v>1</v>
       </c>
       <c r="K11" s="13" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="L11" s="7" t="n">
         <f aca="false">IF(A11="","",IF(K11="50/50",0.5,IF(K11="Prorata salaires",Paramètres!$B$9,IF(K11="Personne 1 seul",1,IF(K11="Personne 2 seul",0,0.5)))))</f>
@@ -2682,16 +2787,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E12" s="18" t="n">
         <v>28</v>
@@ -2701,17 +2806,17 @@
         <v>28</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I12" s="13"/>
       <c r="J12" s="13" t="n">
         <v>8</v>
       </c>
       <c r="K12" s="13" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="L12" s="7" t="n">
         <f aca="false">IF(A12="","",IF(K12="50/50",0.5,IF(K12="Prorata salaires",Paramètres!$B$9,IF(K12="Personne 1 seul",1,IF(K12="Personne 2 seul",0,0.5)))))</f>
@@ -2728,16 +2833,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E13" s="18" t="n">
         <v>600</v>
@@ -2747,15 +2852,15 @@
         <v>600</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I13" s="13"/>
       <c r="J13" s="13"/>
       <c r="K13" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L13" s="7" t="n">
         <f aca="false">IF(A13="","",IF(K13="50/50",0.5,IF(K13="Prorata salaires",Paramètres!$B$9,IF(K13="Personne 1 seul",1,IF(K13="Personne 2 seul",0,0.5)))))</f>
@@ -2772,16 +2877,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E14" s="18" t="n">
         <v>150</v>
@@ -2791,19 +2896,19 @@
         <v>150</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="J14" s="13" t="n">
         <v>3</v>
       </c>
       <c r="K14" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L14" s="7" t="n">
         <f aca="false">IF(A14="","",IF(K14="50/50",0.5,IF(K14="Prorata salaires",Paramètres!$B$9,IF(K14="Personne 1 seul",1,IF(K14="Personne 2 seul",0,0.5)))))</f>
@@ -2820,16 +2925,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E15" s="18" t="n">
         <v>90</v>
@@ -2839,19 +2944,19 @@
         <v>90</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="J15" s="13" t="n">
         <v>28</v>
       </c>
       <c r="K15" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L15" s="7" t="n">
         <f aca="false">IF(A15="","",IF(K15="50/50",0.5,IF(K15="Prorata salaires",Paramètres!$B$9,IF(K15="Personne 1 seul",1,IF(K15="Personne 2 seul",0,0.5)))))</f>
@@ -2868,16 +2973,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="B16" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="B16" s="13" t="s">
-        <v>129</v>
-      </c>
       <c r="C16" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E16" s="18" t="n">
         <v>600</v>
@@ -2887,15 +2992,15 @@
         <v>50</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I16" s="13"/>
       <c r="J16" s="13"/>
       <c r="K16" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L16" s="7" t="n">
         <f aca="false">IF(A16="","",IF(K16="50/50",0.5,IF(K16="Prorata salaires",Paramètres!$B$9,IF(K16="Personne 1 seul",1,IF(K16="Personne 2 seul",0,0.5)))))</f>
@@ -2912,16 +3017,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E17" s="18" t="n">
         <v>30</v>
@@ -2931,15 +3036,15 @@
         <v>30</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I17" s="13"/>
       <c r="J17" s="13"/>
       <c r="K17" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L17" s="7" t="n">
         <f aca="false">IF(A17="","",IF(K17="50/50",0.5,IF(K17="Prorata salaires",Paramètres!$B$9,IF(K17="Personne 1 seul",1,IF(K17="Personne 2 seul",0,0.5)))))</f>
@@ -2956,16 +3061,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E18" s="18" t="n">
         <v>500</v>
@@ -2975,15 +3080,15 @@
         <v>41.6666666666667</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I18" s="13"/>
       <c r="J18" s="13"/>
       <c r="K18" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L18" s="7" t="n">
         <f aca="false">IF(A18="","",IF(K18="50/50",0.5,IF(K18="Prorata salaires",Paramètres!$B$9,IF(K18="Personne 1 seul",1,IF(K18="Personne 2 seul",0,0.5)))))</f>
@@ -3000,16 +3105,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E19" s="21" t="n">
         <f aca="false">Paramètres!$B$22*SUMIFS(Revenus!$F$5:$F$24,Revenus!$B$5:$B$24,"Salaire")</f>
@@ -3020,19 +3125,19 @@
         <v>129</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I19" s="13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="J19" s="13" t="n">
         <v>3</v>
       </c>
       <c r="K19" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L19" s="7" t="n">
         <f aca="false">IF(A19="","",IF(K19="50/50",0.5,IF(K19="Prorata salaires",Paramètres!$B$9,IF(K19="Personne 1 seul",1,IF(K19="Personne 2 seul",0,0.5)))))</f>
@@ -3049,16 +3154,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E20" s="18" t="n">
         <v>50</v>
@@ -3068,19 +3173,19 @@
         <v>50</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I20" s="13" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="J20" s="13" t="n">
         <v>4</v>
       </c>
       <c r="K20" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L20" s="7" t="n">
         <f aca="false">IF(A20="","",IF(K20="50/50",0.5,IF(K20="Prorata salaires",Paramètres!$B$9,IF(K20="Personne 1 seul",1,IF(K20="Personne 2 seul",0,0.5)))))</f>
@@ -3097,16 +3202,16 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E21" s="18" t="n">
         <v>50</v>
@@ -3116,19 +3221,19 @@
         <v>50</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I21" s="13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="J21" s="13" t="n">
         <v>4</v>
       </c>
       <c r="K21" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L21" s="7" t="n">
         <f aca="false">IF(A21="","",IF(K21="50/50",0.5,IF(K21="Prorata salaires",Paramètres!$B$9,IF(K21="Personne 1 seul",1,IF(K21="Personne 2 seul",0,0.5)))))</f>
@@ -3145,16 +3250,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E22" s="18" t="n">
         <v>120</v>
@@ -3164,17 +3269,17 @@
         <v>120</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I22" s="13"/>
       <c r="J22" s="13" t="n">
         <v>1</v>
       </c>
       <c r="K22" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L22" s="7" t="n">
         <f aca="false">IF(A22="","",IF(K22="50/50",0.5,IF(K22="Prorata salaires",Paramètres!$B$9,IF(K22="Personne 1 seul",1,IF(K22="Personne 2 seul",0,0.5)))))</f>
@@ -3191,16 +3296,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E23" s="18" t="n">
         <v>30</v>
@@ -3210,17 +3315,17 @@
         <v>30</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I23" s="13"/>
       <c r="J23" s="13" t="n">
         <v>1</v>
       </c>
       <c r="K23" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L23" s="7" t="n">
         <f aca="false">IF(A23="","",IF(K23="50/50",0.5,IF(K23="Prorata salaires",Paramètres!$B$9,IF(K23="Personne 1 seul",1,IF(K23="Personne 2 seul",0,0.5)))))</f>
@@ -3237,16 +3342,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E24" s="18" t="n">
         <v>60</v>
@@ -3256,15 +3361,15 @@
         <v>60</v>
       </c>
       <c r="G24" s="13" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I24" s="13"/>
       <c r="J24" s="13"/>
       <c r="K24" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L24" s="7" t="n">
         <f aca="false">IF(A24="","",IF(K24="50/50",0.5,IF(K24="Prorata salaires",Paramètres!$B$9,IF(K24="Personne 1 seul",1,IF(K24="Personne 2 seul",0,0.5)))))</f>
@@ -4121,7 +4226,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="22" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F55" s="9" t="n">
         <f aca="false">SUM(F5:F54)</f>
@@ -4188,17 +4293,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>18</v>
@@ -4207,43 +4312,43 @@
         <v>3</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D5" s="18" t="n">
         <v>2400</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F5" s="6" t="n">
         <f aca="false">IF(A5="","",IFERROR(D5/INDEX(Paramètres!$E$4:$E$7,MATCH(E5,Paramètres!$D$4:$D$7,0)),0))</f>
         <v>2400</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H5" s="13" t="n">
         <v>28</v>
@@ -4251,26 +4356,26 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D6" s="18" t="n">
         <v>1900</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F6" s="6" t="n">
         <f aca="false">IF(A6="","",IFERROR(D6/INDEX(Paramètres!$E$4:$E$7,MATCH(E6,Paramètres!$D$4:$D$7,0)),0))</f>
         <v>1900</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H6" s="13" t="n">
         <v>30</v>
@@ -4278,26 +4383,26 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D7" s="18" t="n">
         <v>140</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F7" s="6" t="n">
         <f aca="false">IF(A7="","",IFERROR(D7/INDEX(Paramètres!$E$4:$E$7,MATCH(E7,Paramètres!$D$4:$D$7,0)),0))</f>
         <v>140</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H7" s="13" t="n">
         <v>5</v>
@@ -4305,26 +4410,26 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="B8" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="B8" s="13" t="s">
-        <v>154</v>
-      </c>
       <c r="C8" s="13" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D8" s="18" t="n">
         <v>270</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F8" s="6" t="n">
         <f aca="false">IF(A8="","",IFERROR(D8/INDEX(Paramètres!$E$4:$E$7,MATCH(E8,Paramètres!$D$4:$D$7,0)),0))</f>
         <v>90</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H8" s="13" t="n">
         <v>5</v>
@@ -4540,7 +4645,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="22" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F25" s="9" t="n">
         <f aca="false">SUM(F5:F24)</f>
@@ -4577,7 +4682,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
@@ -4587,59 +4692,63 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="22"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>102</v>
+        <v>104</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E5" s="18" t="n">
         <v>35</v>
@@ -4649,27 +4758,31 @@
         <v>35</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="I5" s="13" t="n">
         <v>10</v>
       </c>
+      <c r="J5" s="5" t="str">
+        <f aca="false">IF(OR($A5="",AND($B5&lt;&gt;Paramètres!$B$4,$B5&lt;&gt;Paramètres!$B$5)),"",IF(IF($B5=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H5&lt;&gt;"",$H5,IF($B5=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v>Compte Alex</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E6" s="18" t="n">
         <v>120</v>
@@ -4679,25 +4792,29 @@
         <v>40</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="H6" s="13" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="I6" s="13"/>
+      <c r="J6" s="5" t="str">
+        <f aca="false">IF(OR($A6="",AND($B6&lt;&gt;Paramètres!$B$4,$B6&lt;&gt;Paramètres!$B$5)),"",IF(IF($B6=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H6&lt;&gt;"",$H6,IF($B6=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v>Compte Alex</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E7" s="18" t="n">
         <v>11</v>
@@ -4707,13 +4824,17 @@
         <v>11</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H7" s="13" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="I7" s="13" t="n">
         <v>15</v>
+      </c>
+      <c r="J7" s="5" t="str">
+        <f aca="false">IF(OR($A7="",AND($B7&lt;&gt;Paramètres!$B$4,$B7&lt;&gt;Paramètres!$B$5)),"",IF(IF($B7=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H7&lt;&gt;"",$H7,IF($B7=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v>Compte Alex</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4729,6 +4850,10 @@
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
       <c r="I8" s="13"/>
+      <c r="J8" s="5" t="str">
+        <f aca="false">IF(OR($A8="",AND($B8&lt;&gt;Paramètres!$B$4,$B8&lt;&gt;Paramètres!$B$5)),"",IF(IF($B8=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H8&lt;&gt;"",$H8,IF($B8=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13"/>
@@ -4743,6 +4868,10 @@
       <c r="G9" s="13"/>
       <c r="H9" s="13"/>
       <c r="I9" s="13"/>
+      <c r="J9" s="5" t="str">
+        <f aca="false">IF(OR($A9="",AND($B9&lt;&gt;Paramètres!$B$4,$B9&lt;&gt;Paramètres!$B$5)),"",IF(IF($B9=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H9&lt;&gt;"",$H9,IF($B9=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13"/>
@@ -4757,6 +4886,10 @@
       <c r="G10" s="13"/>
       <c r="H10" s="13"/>
       <c r="I10" s="13"/>
+      <c r="J10" s="5" t="str">
+        <f aca="false">IF(OR($A10="",AND($B10&lt;&gt;Paramètres!$B$4,$B10&lt;&gt;Paramètres!$B$5)),"",IF(IF($B10=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H10&lt;&gt;"",$H10,IF($B10=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13"/>
@@ -4771,6 +4904,10 @@
       <c r="G11" s="13"/>
       <c r="H11" s="13"/>
       <c r="I11" s="13"/>
+      <c r="J11" s="5" t="str">
+        <f aca="false">IF(OR($A11="",AND($B11&lt;&gt;Paramètres!$B$4,$B11&lt;&gt;Paramètres!$B$5)),"",IF(IF($B11=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H11&lt;&gt;"",$H11,IF($B11=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13"/>
@@ -4785,6 +4922,10 @@
       <c r="G12" s="13"/>
       <c r="H12" s="13"/>
       <c r="I12" s="13"/>
+      <c r="J12" s="5" t="str">
+        <f aca="false">IF(OR($A12="",AND($B12&lt;&gt;Paramètres!$B$4,$B12&lt;&gt;Paramètres!$B$5)),"",IF(IF($B12=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H12&lt;&gt;"",$H12,IF($B12=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13"/>
@@ -4799,6 +4940,10 @@
       <c r="G13" s="13"/>
       <c r="H13" s="13"/>
       <c r="I13" s="13"/>
+      <c r="J13" s="5" t="str">
+        <f aca="false">IF(OR($A13="",AND($B13&lt;&gt;Paramètres!$B$4,$B13&lt;&gt;Paramètres!$B$5)),"",IF(IF($B13=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H13&lt;&gt;"",$H13,IF($B13=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13"/>
@@ -4813,6 +4958,10 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
       <c r="I14" s="13"/>
+      <c r="J14" s="5" t="str">
+        <f aca="false">IF(OR($A14="",AND($B14&lt;&gt;Paramètres!$B$4,$B14&lt;&gt;Paramètres!$B$5)),"",IF(IF($B14=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H14&lt;&gt;"",$H14,IF($B14=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13"/>
@@ -4827,6 +4976,10 @@
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
       <c r="I15" s="13"/>
+      <c r="J15" s="5" t="str">
+        <f aca="false">IF(OR($A15="",AND($B15&lt;&gt;Paramètres!$B$4,$B15&lt;&gt;Paramètres!$B$5)),"",IF(IF($B15=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H15&lt;&gt;"",$H15,IF($B15=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13"/>
@@ -4841,6 +4994,10 @@
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
       <c r="I16" s="13"/>
+      <c r="J16" s="5" t="str">
+        <f aca="false">IF(OR($A16="",AND($B16&lt;&gt;Paramètres!$B$4,$B16&lt;&gt;Paramètres!$B$5)),"",IF(IF($B16=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H16&lt;&gt;"",$H16,IF($B16=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13"/>
@@ -4855,6 +5012,10 @@
       <c r="G17" s="13"/>
       <c r="H17" s="13"/>
       <c r="I17" s="13"/>
+      <c r="J17" s="5" t="str">
+        <f aca="false">IF(OR($A17="",AND($B17&lt;&gt;Paramètres!$B$4,$B17&lt;&gt;Paramètres!$B$5)),"",IF(IF($B17=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H17&lt;&gt;"",$H17,IF($B17=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13"/>
@@ -4869,6 +5030,10 @@
       <c r="G18" s="13"/>
       <c r="H18" s="13"/>
       <c r="I18" s="13"/>
+      <c r="J18" s="5" t="str">
+        <f aca="false">IF(OR($A18="",AND($B18&lt;&gt;Paramètres!$B$4,$B18&lt;&gt;Paramètres!$B$5)),"",IF(IF($B18=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H18&lt;&gt;"",$H18,IF($B18=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13"/>
@@ -4883,6 +5048,10 @@
       <c r="G19" s="13"/>
       <c r="H19" s="13"/>
       <c r="I19" s="13"/>
+      <c r="J19" s="5" t="str">
+        <f aca="false">IF(OR($A19="",AND($B19&lt;&gt;Paramètres!$B$4,$B19&lt;&gt;Paramètres!$B$5)),"",IF(IF($B19=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H19&lt;&gt;"",$H19,IF($B19=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13"/>
@@ -4897,6 +5066,10 @@
       <c r="G20" s="13"/>
       <c r="H20" s="13"/>
       <c r="I20" s="13"/>
+      <c r="J20" s="5" t="str">
+        <f aca="false">IF(OR($A20="",AND($B20&lt;&gt;Paramètres!$B$4,$B20&lt;&gt;Paramètres!$B$5)),"",IF(IF($B20=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H20&lt;&gt;"",$H20,IF($B20=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13"/>
@@ -4911,6 +5084,10 @@
       <c r="G21" s="13"/>
       <c r="H21" s="13"/>
       <c r="I21" s="13"/>
+      <c r="J21" s="5" t="str">
+        <f aca="false">IF(OR($A21="",AND($B21&lt;&gt;Paramètres!$B$4,$B21&lt;&gt;Paramètres!$B$5)),"",IF(IF($B21=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H21&lt;&gt;"",$H21,IF($B21=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13"/>
@@ -4925,6 +5102,10 @@
       <c r="G22" s="13"/>
       <c r="H22" s="13"/>
       <c r="I22" s="13"/>
+      <c r="J22" s="5" t="str">
+        <f aca="false">IF(OR($A22="",AND($B22&lt;&gt;Paramètres!$B$4,$B22&lt;&gt;Paramètres!$B$5)),"",IF(IF($B22=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H22&lt;&gt;"",$H22,IF($B22=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13"/>
@@ -4939,6 +5120,10 @@
       <c r="G23" s="13"/>
       <c r="H23" s="13"/>
       <c r="I23" s="13"/>
+      <c r="J23" s="5" t="str">
+        <f aca="false">IF(OR($A23="",AND($B23&lt;&gt;Paramètres!$B$4,$B23&lt;&gt;Paramètres!$B$5)),"",IF(IF($B23=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H23&lt;&gt;"",$H23,IF($B23=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13"/>
@@ -4953,6 +5138,10 @@
       <c r="G24" s="13"/>
       <c r="H24" s="13"/>
       <c r="I24" s="13"/>
+      <c r="J24" s="5" t="str">
+        <f aca="false">IF(OR($A24="",AND($B24&lt;&gt;Paramètres!$B$4,$B24&lt;&gt;Paramètres!$B$5)),"",IF(IF($B24=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H24&lt;&gt;"",$H24,IF($B24=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13"/>
@@ -4967,6 +5156,10 @@
       <c r="G25" s="13"/>
       <c r="H25" s="13"/>
       <c r="I25" s="13"/>
+      <c r="J25" s="5" t="str">
+        <f aca="false">IF(OR($A25="",AND($B25&lt;&gt;Paramètres!$B$4,$B25&lt;&gt;Paramètres!$B$5)),"",IF(IF($B25=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H25&lt;&gt;"",$H25,IF($B25=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13"/>
@@ -4981,6 +5174,10 @@
       <c r="G26" s="13"/>
       <c r="H26" s="13"/>
       <c r="I26" s="13"/>
+      <c r="J26" s="5" t="str">
+        <f aca="false">IF(OR($A26="",AND($B26&lt;&gt;Paramètres!$B$4,$B26&lt;&gt;Paramètres!$B$5)),"",IF(IF($B26=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H26&lt;&gt;"",$H26,IF($B26=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13"/>
@@ -4995,6 +5192,10 @@
       <c r="G27" s="13"/>
       <c r="H27" s="13"/>
       <c r="I27" s="13"/>
+      <c r="J27" s="5" t="str">
+        <f aca="false">IF(OR($A27="",AND($B27&lt;&gt;Paramètres!$B$4,$B27&lt;&gt;Paramètres!$B$5)),"",IF(IF($B27=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H27&lt;&gt;"",$H27,IF($B27=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13"/>
@@ -5009,6 +5210,10 @@
       <c r="G28" s="13"/>
       <c r="H28" s="13"/>
       <c r="I28" s="13"/>
+      <c r="J28" s="5" t="str">
+        <f aca="false">IF(OR($A28="",AND($B28&lt;&gt;Paramètres!$B$4,$B28&lt;&gt;Paramètres!$B$5)),"",IF(IF($B28=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H28&lt;&gt;"",$H28,IF($B28=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="13"/>
@@ -5023,6 +5228,10 @@
       <c r="G29" s="13"/>
       <c r="H29" s="13"/>
       <c r="I29" s="13"/>
+      <c r="J29" s="5" t="str">
+        <f aca="false">IF(OR($A29="",AND($B29&lt;&gt;Paramètres!$B$4,$B29&lt;&gt;Paramètres!$B$5)),"",IF(IF($B29=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H29&lt;&gt;"",$H29,IF($B29=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13"/>
@@ -5037,6 +5246,10 @@
       <c r="G30" s="13"/>
       <c r="H30" s="13"/>
       <c r="I30" s="13"/>
+      <c r="J30" s="5" t="str">
+        <f aca="false">IF(OR($A30="",AND($B30&lt;&gt;Paramètres!$B$4,$B30&lt;&gt;Paramètres!$B$5)),"",IF(IF($B30=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H30&lt;&gt;"",$H30,IF($B30=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13"/>
@@ -5051,6 +5264,10 @@
       <c r="G31" s="13"/>
       <c r="H31" s="13"/>
       <c r="I31" s="13"/>
+      <c r="J31" s="5" t="str">
+        <f aca="false">IF(OR($A31="",AND($B31&lt;&gt;Paramètres!$B$4,$B31&lt;&gt;Paramètres!$B$5)),"",IF(IF($B31=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H31&lt;&gt;"",$H31,IF($B31=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13"/>
@@ -5065,6 +5282,10 @@
       <c r="G32" s="13"/>
       <c r="H32" s="13"/>
       <c r="I32" s="13"/>
+      <c r="J32" s="5" t="str">
+        <f aca="false">IF(OR($A32="",AND($B32&lt;&gt;Paramètres!$B$4,$B32&lt;&gt;Paramètres!$B$5)),"",IF(IF($B32=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H32&lt;&gt;"",$H32,IF($B32=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13"/>
@@ -5079,6 +5300,10 @@
       <c r="G33" s="13"/>
       <c r="H33" s="13"/>
       <c r="I33" s="13"/>
+      <c r="J33" s="5" t="str">
+        <f aca="false">IF(OR($A33="",AND($B33&lt;&gt;Paramètres!$B$4,$B33&lt;&gt;Paramètres!$B$5)),"",IF(IF($B33=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H33&lt;&gt;"",$H33,IF($B33=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13"/>
@@ -5093,6 +5318,10 @@
       <c r="G34" s="13"/>
       <c r="H34" s="13"/>
       <c r="I34" s="13"/>
+      <c r="J34" s="5" t="str">
+        <f aca="false">IF(OR($A34="",AND($B34&lt;&gt;Paramètres!$B$4,$B34&lt;&gt;Paramètres!$B$5)),"",IF(IF($B34=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H34&lt;&gt;"",$H34,IF($B34=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13"/>
@@ -5107,6 +5336,10 @@
       <c r="G35" s="13"/>
       <c r="H35" s="13"/>
       <c r="I35" s="13"/>
+      <c r="J35" s="5" t="str">
+        <f aca="false">IF(OR($A35="",AND($B35&lt;&gt;Paramètres!$B$4,$B35&lt;&gt;Paramètres!$B$5)),"",IF(IF($B35=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H35&lt;&gt;"",$H35,IF($B35=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13"/>
@@ -5121,6 +5354,10 @@
       <c r="G36" s="13"/>
       <c r="H36" s="13"/>
       <c r="I36" s="13"/>
+      <c r="J36" s="5" t="str">
+        <f aca="false">IF(OR($A36="",AND($B36&lt;&gt;Paramètres!$B$4,$B36&lt;&gt;Paramètres!$B$5)),"",IF(IF($B36=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H36&lt;&gt;"",$H36,IF($B36=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13"/>
@@ -5135,6 +5372,10 @@
       <c r="G37" s="13"/>
       <c r="H37" s="13"/>
       <c r="I37" s="13"/>
+      <c r="J37" s="5" t="str">
+        <f aca="false">IF(OR($A37="",AND($B37&lt;&gt;Paramètres!$B$4,$B37&lt;&gt;Paramètres!$B$5)),"",IF(IF($B37=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H37&lt;&gt;"",$H37,IF($B37=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13"/>
@@ -5149,6 +5390,10 @@
       <c r="G38" s="13"/>
       <c r="H38" s="13"/>
       <c r="I38" s="13"/>
+      <c r="J38" s="5" t="str">
+        <f aca="false">IF(OR($A38="",AND($B38&lt;&gt;Paramètres!$B$4,$B38&lt;&gt;Paramètres!$B$5)),"",IF(IF($B38=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H38&lt;&gt;"",$H38,IF($B38=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="13"/>
@@ -5163,6 +5408,10 @@
       <c r="G39" s="13"/>
       <c r="H39" s="13"/>
       <c r="I39" s="13"/>
+      <c r="J39" s="5" t="str">
+        <f aca="false">IF(OR($A39="",AND($B39&lt;&gt;Paramètres!$B$4,$B39&lt;&gt;Paramètres!$B$5)),"",IF(IF($B39=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H39&lt;&gt;"",$H39,IF($B39=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="13"/>
@@ -5177,6 +5426,10 @@
       <c r="G40" s="13"/>
       <c r="H40" s="13"/>
       <c r="I40" s="13"/>
+      <c r="J40" s="5" t="str">
+        <f aca="false">IF(OR($A40="",AND($B40&lt;&gt;Paramètres!$B$4,$B40&lt;&gt;Paramètres!$B$5)),"",IF(IF($B40=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H40&lt;&gt;"",$H40,IF($B40=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="13"/>
@@ -5191,6 +5444,10 @@
       <c r="G41" s="13"/>
       <c r="H41" s="13"/>
       <c r="I41" s="13"/>
+      <c r="J41" s="5" t="str">
+        <f aca="false">IF(OR($A41="",AND($B41&lt;&gt;Paramètres!$B$4,$B41&lt;&gt;Paramètres!$B$5)),"",IF(IF($B41=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H41&lt;&gt;"",$H41,IF($B41=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="13"/>
@@ -5205,6 +5462,10 @@
       <c r="G42" s="13"/>
       <c r="H42" s="13"/>
       <c r="I42" s="13"/>
+      <c r="J42" s="5" t="str">
+        <f aca="false">IF(OR($A42="",AND($B42&lt;&gt;Paramètres!$B$4,$B42&lt;&gt;Paramètres!$B$5)),"",IF(IF($B42=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H42&lt;&gt;"",$H42,IF($B42=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="13"/>
@@ -5219,6 +5480,10 @@
       <c r="G43" s="13"/>
       <c r="H43" s="13"/>
       <c r="I43" s="13"/>
+      <c r="J43" s="5" t="str">
+        <f aca="false">IF(OR($A43="",AND($B43&lt;&gt;Paramètres!$B$4,$B43&lt;&gt;Paramètres!$B$5)),"",IF(IF($B43=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H43&lt;&gt;"",$H43,IF($B43=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="13"/>
@@ -5233,10 +5498,14 @@
       <c r="G44" s="13"/>
       <c r="H44" s="13"/>
       <c r="I44" s="13"/>
+      <c r="J44" s="5" t="str">
+        <f aca="false">IF(OR($A44="",AND($B44&lt;&gt;Paramètres!$B$4,$B44&lt;&gt;Paramètres!$B$5)),"",IF(IF($B44=Paramètres!$B$4,Paramètres!$B$15,Paramètres!$C$15)="Forfait","",IF($H44&lt;&gt;"",$H44,IF($B44=Paramètres!$B$4,Paramètres!$B$6,Paramètres!$B$7))))</f>
+        <v/>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="22" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F45" s="9" t="n">
         <f aca="false">SUM(F5:F44)</f>
@@ -5245,20 +5514,20 @@
     </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G44" type="list">
-      <formula1>"Prélèvement,Carte,Chèque,Espèces,Virement"</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D44" type="list">
+      <formula1>"Mensuelle,Trimestrielle,Semestrielle,Annuelle"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H44" type="list">
       <formula1>Comptes!$A$5:$A$14</formula1>
       <formula2>0</formula2>
     </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G44" type="list">
+      <formula1>"Prélèvement,Carte,Chèque,Espèces,Virement"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B44" type="list">
       <formula1>Paramètres!$B$4:$B$5</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D44" type="list">
-      <formula1>"Mensuelle,Trimestrielle,Semestrielle,Annuelle"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -5288,17 +5557,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="23" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B4" s="6" t="n">
         <f aca="false">SUMIFS(Charges!$F$5:$F$54,Charges!$B$5:$B$54,"Imprévus")</f>
@@ -5307,7 +5576,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B5" s="24" t="n">
         <v>46266</v>
@@ -5315,7 +5584,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>0</v>
@@ -5323,7 +5592,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B7" s="25" t="n">
         <f aca="true">IF(B5="",0,MAX(0,(YEAR(TODAY())-YEAR(B5))*12+MONTH(TODAY())-MONTH(B5)+1))</f>
@@ -5332,7 +5601,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B8" s="6" t="n">
         <f aca="false">B6+B4*B7</f>
@@ -5341,7 +5610,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">SUM(C13:C62)</f>
@@ -5350,7 +5619,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">B8-B9</f>
@@ -5359,21 +5628,21 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5381,13 +5650,13 @@
         <v>46285</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C13" s="18" t="n">
         <v>220</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5395,13 +5664,13 @@
         <v>46300</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C14" s="18" t="n">
         <v>85</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>